<commit_message>
Actualizacion plantilla de evaluacion
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Grupales/PLANILLA DE EVALUACION FINAL FASE 2.xlsx
+++ b/Fase 2/Evidencias Grupales/PLANILLA DE EVALUACION FINAL FASE 2.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9353449a8f9cae3a/Documentos/DUOC UC/2025/Capstone/Capstone 002/Evaluación N°2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9353449a8f9cae3a/Documentos/DUOC UC/2025/Capstone/Capstone 002/Evaluación N°3/Nueva carpeta/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="633" documentId="8_{2EFDF332-31E9-4C74-A6B5-E695634C1C45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0A21AED6-806A-4BA8-AA3F-CB64C36CFCB8}"/>
+  <xr:revisionPtr revIDLastSave="765" documentId="8_{2EFDF332-31E9-4C74-A6B5-E695634C1C45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54557401-712D-4D9C-B186-A925595518C6}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="EVALUACION2" sheetId="1" r:id="rId1"/>
-    <sheet name="RUBRICA" sheetId="12" r:id="rId2"/>
+    <sheet name="RUBRICA" sheetId="12" r:id="rId1"/>
+    <sheet name="EVALUACION1" sheetId="1" r:id="rId2"/>
     <sheet name="ESCALA_IEP" sheetId="2" state="hidden" r:id="rId3"/>
     <sheet name="ESCALA_PRESENTACION" sheetId="3" state="hidden" r:id="rId4"/>
     <sheet name="ESCALA_TRAB_EQUIP" sheetId="4" state="hidden" r:id="rId5"/>
@@ -45,8 +45,11 @@
     <definedName name="RE_TL">'RELEVANCIA-PUNTAJE'!$B$4</definedName>
     <definedName name="TL">'RELEVANCIA-PUNTAJE'!$B$2</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191028"/>
   <extLst>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
+      <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
@@ -63,49 +66,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="65">
-  <si>
-    <t>PUNTOS</t>
-  </si>
-  <si>
-    <t>NOTA</t>
-  </si>
-  <si>
-    <t>INTEGRANTES</t>
-  </si>
-  <si>
-    <t>Relevancia</t>
-  </si>
-  <si>
-    <t>Puntaje</t>
-  </si>
-  <si>
-    <t>Completamente logrado</t>
-  </si>
-  <si>
-    <t>Logrado</t>
-  </si>
-  <si>
-    <t>No logrado</t>
-  </si>
-  <si>
-    <t>Muy Relevante</t>
-  </si>
-  <si>
-    <t>GRUPAL</t>
-  </si>
-  <si>
-    <t>Nivel de Logro</t>
-  </si>
-  <si>
-    <t>NIVELES DE LOGRO Y PUNTAJES</t>
-  </si>
-  <si>
-    <t>Aspectos a Evaluar</t>
-  </si>
-  <si>
-    <t>Nota</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="79">
   <si>
     <t>Indicador de Evaluación</t>
   </si>
@@ -114,6 +75,21 @@
   </si>
   <si>
     <t>Ponderación del Indicador de Evaluación</t>
+  </si>
+  <si>
+    <r>
+      <t>Completamente Logrado</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">  (100%)</t>
+    </r>
   </si>
   <si>
     <r>
@@ -134,106 +110,70 @@
     <t xml:space="preserve">Logro incipiente </t>
   </si>
   <si>
-    <t>El texto presenta de 1 a 5 errores de ortografía, redacción o en las citas y referencias del informe.</t>
+    <t>No logrado</t>
   </si>
   <si>
-    <t>El texto presenta de 6 a 10 errores de ortografía, redacción o en las citas y referencias del informe.</t>
+    <t>1. Implementa una metodología que permite el logro de los objetivos propuestos, de acuerdo a los estándares de la disciplina.</t>
   </si>
   <si>
-    <t>El texto presenta más de 10 errores de ortografía, redacción o en las citas y referencias del informe.</t>
+    <t xml:space="preserve">Describe la metodología utilizada de acuerdo a los estándares de la disciplina, alcanzando todos los objetivos propuestos para el proyecto. </t>
   </si>
   <si>
-    <t>El texto cumple con las reglas ortografía y de redacción en todos sus apartados y utiliza correctamente todas las normas de citación y referencias.</t>
+    <t xml:space="preserve">Describe la metodología utilizada de acuerdo a los estándares de la disciplina, pero cumple parcialmente los objetivos propuestos para el proyecto. </t>
   </si>
   <si>
-    <t>Logro Incipiente</t>
+    <t xml:space="preserve">Describe la metodología utilizada cumpliendo parcialmente con los estándares de la disciplina y con los objetivos propuestos para el proyecto. </t>
   </si>
   <si>
-    <t>Logro incipiente</t>
+    <t xml:space="preserve">Describe la metodología utilizada sin cumplir los estándares de la disciplina ni los objetivos propuestos para el proyecto. </t>
   </si>
   <si>
-    <r>
-      <t>Completamente Logrado</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">  (100%)</t>
-    </r>
+    <t>2. Genera evidencias que dan cuenta del cumplimiento del Proyecto CAPSTONE, en relación a documentación, programación y almacenamiento de datos, de acuerdo a lo planificado por el equipo y que cumpla con estándares de desarrollo de la industria</t>
   </si>
   <si>
-    <t xml:space="preserve">1. Propone ajustes al Proyecto APT considerando dificultades, facilitadores y retroalimentación. </t>
+    <t>Genera evidencias que dan cuenta del cumplimiento del Proyecto CAPSTONE, en relación a documentación, programación y almacenamiento de datos, de acuerdo a lo planificado por el equipo y que cumpla con estándares de desarrollo de la industria</t>
   </si>
   <si>
-    <t>Señala los ajustes que realizó o realizará y los justifica considerando las dificultades, facilitadores y retroalimentación del docente.</t>
+    <t>Genera evidencias que dan cuenta del cumplimiento del Proyecto CAPSTONE, en relación a documentación, programación y almacenamiento de datos, de acuerdo a lo planificado por el equipo y no cumplen con estándares de desarrollo de la industria</t>
   </si>
   <si>
-    <t>Señala algunos de los ajustes que realizó o realizará y los justifica considerando las dificultades, facilitadores o retroalimentación del docente.</t>
+    <t>Genera evidencias pero ellas no dan cuenta del cumplimiento del Proyecto CAPSTONE, en relación a documentación, programación y almacenamiento de datos, de acuerdo a lo planificado por el equipo, pero si cumple con estándares de desarrollo de la industria</t>
   </si>
   <si>
-    <t>Señala los ajustes que realizó o realizará, pero no los justifica.</t>
+    <t>Genera evidencias pero ellas no dan cuenta del cumplimiento del Proyecto CAPSTONE, en relación a documentación, programación y almacenamiento de datos, de acuerdo a lo planificado por el equipo, y no cumplen con estándares de desarrollo de la industria</t>
   </si>
   <si>
-    <t>No incluye ajustes ni justifica por qué mantiene su plan inicial.</t>
+    <t>3. Relaciona el Proyecto APT con sus intereses profesionales. *</t>
   </si>
   <si>
-    <t>2. Aplica una metodología que permite el logro de los objetivos propuestos, de acuerdo a los estándares de la disciplina.</t>
+    <t xml:space="preserve">Menciona los intereses profesionales y explica con claridad cómo estos se ven reflejados en el proyecto. </t>
   </si>
   <si>
-    <t xml:space="preserve">Aplica la metodología definida de acuerdo a los estándares de la disciplina, pero no se observa el cumplimiento de objetivos propuestos para el avance del proyecto. </t>
+    <t>Menciona los intereses profesionales, pero no queda completamente clara su conexión con el proyecto.</t>
   </si>
   <si>
-    <t xml:space="preserve">Aplica la metodología definida cumpliendo parcialmente con los estándares de la disciplina y con los objetivos propuestos para el avance del proyecto. </t>
+    <t xml:space="preserve">Menciona los intereses profesionales sin conectarlos con el proyecto. </t>
   </si>
   <si>
-    <t xml:space="preserve">Aplica la metodología definida sin cumplir los estándares de la disciplina ni los objetivos propuestos para el avance del proyecto. </t>
+    <t>No menciona los intereses profesionales.</t>
   </si>
   <si>
-    <t xml:space="preserve">5. Utiliza reglas de redacción, ortografía (literal, puntual, acentual) y las normas para citas y referencias. </t>
+    <t>4. Relaciona el Proyecto APT con las competencias del perfil de egreso de su Plan de Estudio.</t>
   </si>
   <si>
-    <t>8. Demuestra un trabajo en equipo en donde todos los miembros del equipo expresan con fluidez el conocimiento del tema expuesto y  participan de las actividades planificadas en el proyecto</t>
+    <t xml:space="preserve">Describe una relación coherente entre el proyecto y el perfil de egreso del plan de estudio, especificando cómo debe utilizar distintas competencias para desarrollar su Proyecto APT. </t>
   </si>
   <si>
-    <t>Demuestra un trabajo en equipo en donde todos los miembros del equipo expresan con fluidez el conocimiento del tema expuesto y  participan de las actividades planificadas en el proyecto</t>
+    <t>Describe una relación coherente entre el proyecto y el perfil de egreso del plan de estudio, pero no especifica cómo debe utilizar distintas competencias para desarrollar su Proyecto APT.</t>
   </si>
   <si>
-    <t>Demuestra un trabajo en equipo de manera parcial, en donde todos los miembros del equipo expresan con fluidez el conocimiento del tema expuesto, pero no todos participan de manera equitativa de las actividades planificadas en el proyecto</t>
+    <t>Describe una relación que tiene elementos pero que no son coherentes entre el proyecto y el perfil de egreso del plan de estudio.</t>
   </si>
   <si>
-    <t>Demuestra de manera deficiente el trabajo en equipo en donde los integrantes expresan con poca fluidez y de manera imparcial el conocimiento del tema expuesto y no todos sus miembros participan de manera equitativa de las actividades planificadas en el proyecto</t>
+    <t xml:space="preserve">Describe una relación sin coherencia entre el proyecto y el perfil de egreso del plan de estudio o no relaciona el proyecto con el perfil de egreso. </t>
   </si>
   <si>
-    <t xml:space="preserve">No demuestran un trabajo en equipo, evidenciando en su presentación la nula colaboración de alguno de sus integrantes. </t>
-  </si>
-  <si>
-    <t>X</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Aplica la metodología definida por el equipo de acuerdo a los estándares de la disciplina, alcanzando los objetivos propuestos para el avance del proyecto. </t>
-  </si>
-  <si>
-    <t>3. Genera evidencias que dan cuenta del avance del Proyecto APT en relación a documentación, programación y almacenamiento de datos , de acuerdo a lo planificado por el equipo y que cumpla con estándares de desarrollo de la industria</t>
-  </si>
-  <si>
-    <t>Presenta evidencias de avance que cumplen con lo planificado por el equipo en relación a documentación, programación y almacenamiento de datos, entregando evidencias que cumplan con estándares de desarrollo que actualmente se encuentran presentes en la industria</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Presenta evidencias de avance sin cumplir con lo planificado por el equipo en relación a documentación, programación y almacenamiento de datos, pero si sus entregas evidencian el cumplimiento de estándares de desarrollo que actualmente se encuentran presentes en la industria. </t>
-  </si>
-  <si>
-    <t>Presenta evidencias de avance que cumplen con lo planificado por el equipo en relación a documentación, programación y almacenamiento de datos, entregando evidencias que no cumplen con estándares de desarrollo que actualmente se encuentran presentes en la industria</t>
-  </si>
-  <si>
-    <t>Presenta evidencias de avance sin cumplir con lo planificado por el equipo en relación a documentación, programación y almacenamiento de datos y las evidencias no cumplen con estándares de desarrollo que actualmente se encuentran presentes en la industria</t>
-  </si>
-  <si>
-    <t>4. Utiliza de manera precisa el lenguaje técnico en los entregables de acuerdo con lo requerido por la disciplina.</t>
+    <t>5. Utiliza de manera precisa el lenguaje técnico en los entregables de acuerdo con lo requerido por la disciplina.</t>
   </si>
   <si>
     <t xml:space="preserve">Utiliza lenguaje técnico de su disciplina en todos los entregables de avance del proyecto. </t>
@@ -248,7 +188,22 @@
     <t xml:space="preserve">No utiliza lenguaje técnico de su disciplina en los entregables de avance del proyecto. </t>
   </si>
   <si>
-    <t>6. Entrega la documentación y evidencias requerida por la asignatura de acuerdo a la estrucutra y nombres solicitados, guardando todas las evidencias de avances en Git</t>
+    <t xml:space="preserve">6. Utiliza correctamente las reglas de redacción, ortografía (literal, puntual, acentual) y las normas para citas y referencias. </t>
+  </si>
+  <si>
+    <t>El texto cumple con las reglas ortografía y de redacción en todos sus apartados y utiliza correctamente todas las normas de citación y referencias.</t>
+  </si>
+  <si>
+    <t>El texto presenta de 1 a 5 errores de ortografía, redacción o en las citas y referencias del informe.</t>
+  </si>
+  <si>
+    <t>El texto presenta de 6 a 10 errores de ortografía, redacción o en las citas y referencias del informe.</t>
+  </si>
+  <si>
+    <t>El texto presenta más de 10 errores de ortografía, redacción o en las citas y referencias del informe.</t>
+  </si>
+  <si>
+    <t>7. Entrega la documentación y evidencias requerida por la asignatura de acuerdo a la estrucutra y nombres solicitados, guardando todas las evidencias de avances en Git</t>
   </si>
   <si>
     <t>Entrega la documentación y evidencias requeridas por la asignatura de acuerdo a la estrucutra y nombres solicitados, guardando todas las evidencias de avances en Git</t>
@@ -263,7 +218,22 @@
     <t>No entrega a través de Git la documentación y evidencias de avance requeridas por la asignatura</t>
   </si>
   <si>
-    <t>7.- Generan evidencias claras dentro del repositorio  del aporte de cada uno de los integrantes del equipo que permitan identificar la equidad en el trabajo y la participación de cada estudiante.</t>
+    <t>8. Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información. *</t>
+  </si>
+  <si>
+    <t>Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información en todo momento</t>
+  </si>
+  <si>
+    <t>Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información la mayoría del tiempo.</t>
+  </si>
+  <si>
+    <t>Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información la mitad del tiempo.</t>
+  </si>
+  <si>
+    <t>Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información en menos de la mitad del tiempo.</t>
+  </si>
+  <si>
+    <t>9.-Generan evidencias claras dentro del repositorio  del aporte de cada uno de los integrantes del equipo que permitan identificar la equidad en el trabajo y la participación de cada estudiante.</t>
   </si>
   <si>
     <t>Generan evidencias dentro del repositorio  del proyecto del aporte de cada uno de los integrantes del equipo que permitan identificar la equidad en el trabajo y la participación de cada estudiante</t>
@@ -278,10 +248,85 @@
     <t>No generan evidencias dentro del repositorio  del proyecto del aporte de cada uno de los integrantes del equipo por lo que no se permite identificar la equidad en el trabajo y la participación de cada estudiante</t>
   </si>
   <si>
+    <t>10. Colaboración y trabajo en equipo *</t>
+  </si>
+  <si>
+    <t>El estudiante realiza un excelente trabajo en equipo, fomentando un ambiente positivo, siendo participativo con su equipo en las sesiones presenciales de la asignatura y participando de manera equitativa en la presentación del caso</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El estudiante realiza un buen trabajo en equipo, fomentando un ambiente positivo, siendo participativo con su equipo en las sesiones presenciales de la asignatura, pero no demuestra una participación de manera equitativa en la presentación del caso </t>
+  </si>
+  <si>
+    <t>El estudiante realiza un trabajo deficiente con el equipo, fomentando un ambiente positivo pero no demuestra ser participativo con su equipo en las sesiones presenciales de la asignatura o se ausenta constantemente y/o  no demuestra una participación de manera equitativa en la presentación del caso</t>
+  </si>
+  <si>
+    <t>El estudiante realiza un mal trabajo con el equipo no fomentando un ambiente positivo, no demuestra ser participativo con su equipo en las sesiones presenciales de la asignatura o se ausenta constantemente y no demuestra una participación de manera equitativa en la presentación del caso</t>
+  </si>
+  <si>
+    <t>INTEGRANTES</t>
+  </si>
+  <si>
+    <t>GRUPAL</t>
+  </si>
+  <si>
+    <t>INDIVIDUAL</t>
+  </si>
+  <si>
+    <t>Nivel de Logro</t>
+  </si>
+  <si>
+    <t>NIVELES DE LOGRO Y PUNTAJES</t>
+  </si>
+  <si>
+    <t>Aspectos a Evaluar</t>
+  </si>
+  <si>
+    <t>Completamente logrado</t>
+  </si>
+  <si>
+    <t>Logrado</t>
+  </si>
+  <si>
+    <t>Logro Incipiente</t>
+  </si>
+  <si>
+    <t>Puntaje</t>
+  </si>
+  <si>
+    <t>Nota</t>
+  </si>
+  <si>
+    <t>NOMBRE ALUMNO</t>
+  </si>
+  <si>
+    <t>Capacidad de Trabajo en Equipo</t>
+  </si>
+  <si>
+    <t>PUNTAJE</t>
+  </si>
+  <si>
+    <t>PUNTOS</t>
+  </si>
+  <si>
+    <t>NOTA</t>
+  </si>
+  <si>
+    <t>Relevancia</t>
+  </si>
+  <si>
+    <t>Logro incipiente</t>
+  </si>
+  <si>
+    <t>Muy Relevante</t>
+  </si>
+  <si>
     <t>Esteban Fierro</t>
   </si>
   <si>
     <t>Francisca Herrera</t>
+  </si>
+  <si>
+    <t>X</t>
   </si>
 </sst>
 </file>
@@ -291,7 +336,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="0.0"/>
   </numFmts>
-  <fonts count="18" x14ac:knownFonts="1">
+  <fonts count="17" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -340,6 +385,11 @@
       <name val="Calibri"/>
     </font>
     <font>
+      <sz val="16"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+    </font>
+    <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
@@ -367,13 +417,6 @@
       <family val="2"/>
     </font>
     <font>
-      <b/>
-      <sz val="10"/>
-      <color rgb="FF3B3838"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -387,19 +430,13 @@
       <family val="2"/>
     </font>
     <font>
-      <sz val="9"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="10">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -410,6 +447,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="FFECECEC"/>
         <bgColor rgb="FFECECEC"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDEEAF6"/>
+        <bgColor rgb="FFDEEAF6"/>
       </patternFill>
     </fill>
     <fill>
@@ -432,12 +475,24 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="FFE2EFD9"/>
+        <bgColor rgb="FFE2EFD9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="FF262626"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF92D050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="28">
+  <borders count="29">
     <border>
       <left/>
       <right/>
@@ -589,17 +644,6 @@
     </border>
     <border>
       <left/>
-      <right style="medium">
-        <color rgb="FF000000"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF000000"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right/>
       <top style="thin">
         <color rgb="FF000000"/>
@@ -634,27 +678,65 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FF7F7F7F"/>
+      <left style="thin">
+        <color rgb="FF000000"/>
       </left>
-      <right style="medium">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top style="medium">
-        <color rgb="FF7F7F7F"/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
       </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
-        <color rgb="FF7F7F7F"/>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
       </left>
-      <right style="medium">
-        <color rgb="FF7F7F7F"/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
       </right>
       <top/>
-      <bottom/>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -675,53 +757,7 @@
       <right style="medium">
         <color rgb="FF7F7F7F"/>
       </right>
-      <top style="medium">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color rgb="FF7F7F7F"/>
-      </top>
-      <bottom style="medium">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF7F7F7F"/>
-      </right>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color rgb="FF7F7F7F"/>
-      </right>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FF7F7F7F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color rgb="FF7F7F7F"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color rgb="FF7F7F7F"/>
-      </top>
       <bottom style="medium">
         <color rgb="FF7F7F7F"/>
       </bottom>
@@ -752,15 +788,33 @@
       <diagonal/>
     </border>
     <border>
-      <left/>
+      <left style="medium">
+        <color rgb="FF7F7F7F"/>
+      </left>
       <right style="medium">
         <color rgb="FF7F7F7F"/>
       </right>
       <top style="medium">
         <color rgb="FF7F7F7F"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF7F7F7F"/>
       </bottom>
       <diagonal/>
     </border>
@@ -768,7 +822,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="73">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -781,142 +835,172 @@
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="9" fontId="10" fillId="8" borderId="24" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="14" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="9" fillId="6" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="28" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="9" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="27" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="8" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="255"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="2" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="255"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
@@ -1250,8 +1334,271 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B396D1B-8A63-4A90-BA20-D34AC13A3962}">
+  <dimension ref="A1:F13"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="6" width="38.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A1" s="51" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="51" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="51"/>
+      <c r="D1" s="51"/>
+      <c r="E1" s="51"/>
+      <c r="F1" s="51" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A2" s="51"/>
+      <c r="B2" s="52" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" s="52" t="s">
+        <v>4</v>
+      </c>
+      <c r="D2" s="35" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="34" t="s">
+        <v>6</v>
+      </c>
+      <c r="F2" s="51"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A3" s="51"/>
+      <c r="B3" s="52"/>
+      <c r="C3" s="52"/>
+      <c r="D3" s="36">
+        <v>-0.3</v>
+      </c>
+      <c r="E3" s="36">
+        <v>0</v>
+      </c>
+      <c r="F3" s="51"/>
+    </row>
+    <row r="4" spans="1:6" ht="51" x14ac:dyDescent="0.25">
+      <c r="A4" s="37" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="37" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="37" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="37" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="37" t="s">
+        <v>11</v>
+      </c>
+      <c r="F4" s="38">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" ht="76.5" x14ac:dyDescent="0.25">
+      <c r="A5" s="41" t="s">
+        <v>12</v>
+      </c>
+      <c r="B5" s="37" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="37" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="37" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="37" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="38">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" ht="39" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="41" t="s">
+        <v>17</v>
+      </c>
+      <c r="B6" s="37" t="s">
+        <v>18</v>
+      </c>
+      <c r="C6" s="37" t="s">
+        <v>19</v>
+      </c>
+      <c r="D6" s="37" t="s">
+        <v>20</v>
+      </c>
+      <c r="E6" s="37" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" s="38">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" ht="63.75" x14ac:dyDescent="0.25">
+      <c r="A7" s="42" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="43" t="s">
+        <v>23</v>
+      </c>
+      <c r="C7" s="43" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" s="43" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" s="44" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" s="38">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" ht="38.25" x14ac:dyDescent="0.25">
+      <c r="A8" s="41" t="s">
+        <v>27</v>
+      </c>
+      <c r="B8" s="37" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" s="37" t="s">
+        <v>29</v>
+      </c>
+      <c r="D8" s="37" t="s">
+        <v>30</v>
+      </c>
+      <c r="E8" s="37" t="s">
+        <v>31</v>
+      </c>
+      <c r="F8" s="38">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" ht="51" x14ac:dyDescent="0.25">
+      <c r="A9" s="41" t="s">
+        <v>32</v>
+      </c>
+      <c r="B9" s="37" t="s">
+        <v>33</v>
+      </c>
+      <c r="C9" s="37" t="s">
+        <v>34</v>
+      </c>
+      <c r="D9" s="37" t="s">
+        <v>35</v>
+      </c>
+      <c r="E9" s="37" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9" s="38">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" ht="51" x14ac:dyDescent="0.25">
+      <c r="A10" s="41" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" s="37" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="37" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" s="37" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="37" t="s">
+        <v>41</v>
+      </c>
+      <c r="F10" s="38">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="45" t="s">
+        <v>42</v>
+      </c>
+      <c r="B11" s="26" t="s">
+        <v>43</v>
+      </c>
+      <c r="C11" s="26" t="s">
+        <v>44</v>
+      </c>
+      <c r="D11" s="26" t="s">
+        <v>45</v>
+      </c>
+      <c r="E11" s="46" t="s">
+        <v>46</v>
+      </c>
+      <c r="F11" s="38">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" ht="64.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="47" t="s">
+        <v>47</v>
+      </c>
+      <c r="B12" s="48" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="48" t="s">
+        <v>49</v>
+      </c>
+      <c r="D12" s="48" t="s">
+        <v>50</v>
+      </c>
+      <c r="E12" s="48" t="s">
+        <v>51</v>
+      </c>
+      <c r="F12" s="49">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" ht="90" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="25" t="s">
+        <v>52</v>
+      </c>
+      <c r="B13" s="26" t="s">
+        <v>53</v>
+      </c>
+      <c r="C13" s="26" t="s">
+        <v>54</v>
+      </c>
+      <c r="D13" s="26" t="s">
+        <v>55</v>
+      </c>
+      <c r="E13" s="26" t="s">
+        <v>56</v>
+      </c>
+      <c r="F13" s="38">
+        <v>10</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="5">
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="B1:E1"/>
+    <mergeCell ref="F1:F3"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A2:K895"/>
+  <dimension ref="A2:K926"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1" outlineLevelRow="1" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.7109375" customWidth="1"/>
@@ -1268,27 +1615,45 @@
   <sheetData>
     <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="C2" s="2">
+        <v>0.75</v>
+      </c>
+      <c r="D2" s="2">
+        <v>0.25</v>
+      </c>
+      <c r="E2" s="68">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" ht="30" x14ac:dyDescent="0.25">
       <c r="B3" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" s="33" t="s">
-        <v>9</v>
-      </c>
+        <v>57</v>
+      </c>
+      <c r="C3" s="39" t="s">
+        <v>58</v>
+      </c>
+      <c r="D3" s="40" t="s">
+        <v>59</v>
+      </c>
+      <c r="E3" s="54"/>
     </row>
     <row r="4" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>1</v>
       </c>
-      <c r="B4" s="25" t="s">
-        <v>63</v>
+      <c r="B4" s="27" t="s">
+        <v>76</v>
       </c>
       <c r="C4" s="5">
-        <f>EVALUACION2!$C$22</f>
-        <v>6.3</v>
+        <f>EVALUACION1!$C$21</f>
+        <v>4.8</v>
+      </c>
+      <c r="D4" s="5">
+        <f>$C$32</f>
+        <v>5.8</v>
+      </c>
+      <c r="E4" s="6">
+        <f>C4*C$2+D4*D$2</f>
+        <v>5.05</v>
       </c>
       <c r="G4" s="1"/>
     </row>
@@ -1296,12 +1661,20 @@
       <c r="A5" s="4">
         <v>2</v>
       </c>
-      <c r="B5" s="25" t="s">
-        <v>64</v>
+      <c r="B5" s="27" t="s">
+        <v>77</v>
       </c>
       <c r="C5" s="5">
-        <f>EVALUACION2!$C$22</f>
-        <v>6.3</v>
+        <f>EVALUACION1!$C$21</f>
+        <v>4.8</v>
+      </c>
+      <c r="D5" s="5">
+        <f>C44</f>
+        <v>5.8</v>
+      </c>
+      <c r="E5" s="6">
+        <f t="shared" ref="E5:E6" si="0">C5*C$2+D5*D$2</f>
+        <v>5.05</v>
       </c>
       <c r="G5" s="1"/>
     </row>
@@ -1309,480 +1682,1110 @@
       <c r="A6" s="4">
         <v>3</v>
       </c>
-      <c r="B6" s="25"/>
-      <c r="C6" s="5">
-        <f>EVALUACION2!$C$22</f>
-        <v>6.3</v>
-      </c>
+      <c r="B6" s="27"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="6"/>
       <c r="G6" s="1"/>
     </row>
     <row r="11" spans="1:11" ht="18.75" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="40" t="s">
-        <v>9</v>
+      <c r="A11" s="69" t="s">
+        <v>58</v>
       </c>
       <c r="B11" s="14"/>
-      <c r="C11" s="44" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" s="45" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" s="47"/>
-      <c r="F11" s="47"/>
-      <c r="G11" s="47"/>
-      <c r="H11" s="47"/>
-      <c r="I11" s="47"/>
-      <c r="J11" s="47"/>
-      <c r="K11" s="46"/>
+      <c r="C11" s="61" t="s">
+        <v>60</v>
+      </c>
+      <c r="D11" s="62" t="s">
+        <v>61</v>
+      </c>
+      <c r="E11" s="63"/>
+      <c r="F11" s="63"/>
+      <c r="G11" s="63"/>
+      <c r="H11" s="63"/>
+      <c r="I11" s="63"/>
+      <c r="J11" s="63"/>
+      <c r="K11" s="64"/>
     </row>
     <row r="12" spans="1:11" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="41"/>
-      <c r="B12" s="20" t="s">
-        <v>12</v>
-      </c>
-      <c r="C12" s="43"/>
-      <c r="D12" s="45" t="s">
-        <v>5</v>
-      </c>
-      <c r="E12" s="46"/>
-      <c r="F12" s="45" t="s">
+      <c r="A12" s="67"/>
+      <c r="B12" s="24" t="s">
+        <v>62</v>
+      </c>
+      <c r="C12" s="54"/>
+      <c r="D12" s="62" t="s">
+        <v>63</v>
+      </c>
+      <c r="E12" s="64"/>
+      <c r="F12" s="62" t="s">
+        <v>64</v>
+      </c>
+      <c r="G12" s="64"/>
+      <c r="H12" s="65" t="s">
+        <v>65</v>
+      </c>
+      <c r="I12" s="64"/>
+      <c r="J12" s="62" t="s">
         <v>6</v>
       </c>
-      <c r="G12" s="46"/>
-      <c r="H12" s="48" t="s">
-        <v>23</v>
-      </c>
-      <c r="I12" s="46"/>
-      <c r="J12" s="45" t="s">
-        <v>7</v>
-      </c>
-      <c r="K12" s="46"/>
+      <c r="K12" s="64"/>
     </row>
     <row r="13" spans="1:11" ht="24" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="42"/>
-      <c r="B13" s="28" t="str">
+      <c r="A13" s="70"/>
+      <c r="B13" s="30" t="str">
         <f>RUBRICA!A4</f>
-        <v xml:space="preserve">1. Propone ajustes al Proyecto APT considerando dificultades, facilitadores y retroalimentación. </v>
-      </c>
-      <c r="C13" s="26" t="s">
-        <v>5</v>
-      </c>
-      <c r="D13" s="15" t="str">
-        <f t="shared" ref="D13:D17" si="0">IF($C13=CL,"X","")</f>
-        <v>X</v>
-      </c>
-      <c r="E13" s="15">
+        <v>1. Implementa una metodología que permite el logro de los objetivos propuestos, de acuerdo a los estándares de la disciplina.</v>
+      </c>
+      <c r="C13" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="D13" s="16"/>
+      <c r="E13" s="16" t="str">
         <f>IF(D13="X",100*0.1,"")</f>
-        <v>10</v>
-      </c>
-      <c r="F13" s="15" t="str">
-        <f t="shared" ref="F13:F17" si="1">IF($C13=L,"X","")</f>
         <v/>
       </c>
-      <c r="G13" s="15" t="str">
+      <c r="F13" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="G13" s="16">
         <f>IF(F13="X",60*0.1,"")</f>
+        <v>6</v>
+      </c>
+      <c r="H13" s="16" t="str">
+        <f t="shared" ref="H13:H16" si="1">IF($C13=ML,"X","")</f>
         <v/>
       </c>
-      <c r="H13" s="15" t="str">
-        <f t="shared" ref="H13:H17" si="2">IF($C13=ML,"X","")</f>
-        <v/>
-      </c>
-      <c r="I13" s="15" t="str">
+      <c r="I13" s="16" t="str">
         <f>IF(H13="X",30*0.1,"")</f>
         <v/>
       </c>
-      <c r="J13" s="15" t="str">
-        <f t="shared" ref="J13:J17" si="3">IF($C13=NL,"X","")</f>
+      <c r="J13" s="16" t="str">
+        <f t="shared" ref="J13:J16" si="2">IF($C13=NL,"X","")</f>
         <v/>
       </c>
-      <c r="K13" s="15" t="str">
-        <f t="shared" ref="K13:K17" si="4">IF($J13="X",0,"")</f>
+      <c r="K13" s="16" t="str">
+        <f t="shared" ref="K13:K16" si="3">IF($J13="X",0,"")</f>
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:11" ht="26.45" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="42"/>
-      <c r="B14" s="28" t="str">
+    <row r="14" spans="1:11" ht="48" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="A14" s="70"/>
+      <c r="B14" s="30" t="str">
         <f>RUBRICA!A5</f>
-        <v>2. Aplica una metodología que permite el logro de los objetivos propuestos, de acuerdo a los estándares de la disciplina.</v>
-      </c>
-      <c r="C14" s="26" t="s">
-        <v>5</v>
-      </c>
-      <c r="D14" s="15" t="str">
-        <f t="shared" si="0"/>
-        <v>X</v>
-      </c>
-      <c r="E14" s="15">
-        <f>IF(D14="X",100*0.1,"")</f>
-        <v>10</v>
-      </c>
-      <c r="F14" s="15" t="str">
+        <v>2. Genera evidencias que dan cuenta del cumplimiento del Proyecto CAPSTONE, en relación a documentación, programación y almacenamiento de datos, de acuerdo a lo planificado por el equipo y que cumpla con estándares de desarrollo de la industria</v>
+      </c>
+      <c r="C14" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16" t="str">
+        <f>IF(D14="X",100*0.2,"")</f>
+        <v/>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="G14" s="16">
+        <f>IF(F14="X",60*0.2,"")</f>
+        <v>12</v>
+      </c>
+      <c r="H14" s="16" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="G14" s="15" t="str">
-        <f>IF(F14="X",60*0.1,"")</f>
+      <c r="I14" s="16" t="str">
+        <f>IF(H14="X",30*0.2,"")</f>
         <v/>
       </c>
-      <c r="H14" s="15" t="str">
+      <c r="J14" s="16" t="str">
         <f t="shared" si="2"/>
         <v/>
       </c>
-      <c r="I14" s="15" t="str">
-        <f>IF(H14="X",30*0.1,"")</f>
-        <v/>
-      </c>
-      <c r="J14" s="15" t="str">
+      <c r="K14" s="16" t="str">
         <f t="shared" si="3"/>
         <v/>
       </c>
-      <c r="K14" s="15" t="str">
+    </row>
+    <row r="15" spans="1:11" ht="24" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="A15" s="70"/>
+      <c r="B15" s="30" t="str">
+        <f>RUBRICA!A7</f>
+        <v>4. Relaciona el Proyecto APT con las competencias del perfil de egreso de su Plan de Estudio.</v>
+      </c>
+      <c r="C15" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16" t="str">
+        <f>IF(D15="X",100*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="F15" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="G15" s="16">
+        <f>IF(F15="X",60*0.05,"")</f>
+        <v>3</v>
+      </c>
+      <c r="H15" s="16" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="I15" s="16" t="str">
+        <f>IF(H15="X",30*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="J15" s="16" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="K15" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="16" spans="1:11" ht="24" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="A16" s="70"/>
+      <c r="B16" s="30" t="str">
+        <f>RUBRICA!A8</f>
+        <v>5. Utiliza de manera precisa el lenguaje técnico en los entregables de acuerdo con lo requerido por la disciplina.</v>
+      </c>
+      <c r="C16" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16" t="str">
+        <f>IF(D16="X",100*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="F16" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="G16" s="16">
+        <f>IF(F16="X",60*0.05,"")</f>
+        <v>3</v>
+      </c>
+      <c r="H16" s="16" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+      <c r="I16" s="16" t="str">
+        <f>IF(H16="X",30*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="J16" s="16" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="K16" s="16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="17" spans="1:11" ht="24" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="A17" s="70"/>
+      <c r="B17" s="30" t="str">
+        <f>RUBRICA!A9</f>
+        <v xml:space="preserve">6. Utiliza correctamente las reglas de redacción, ortografía (literal, puntual, acentual) y las normas para citas y referencias. </v>
+      </c>
+      <c r="C17" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="D17" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="E17" s="16">
+        <f>IF(D17="X",100*0.05,"")</f>
+        <v>5</v>
+      </c>
+      <c r="F17" s="16"/>
+      <c r="G17" s="16" t="str">
+        <f>IF(F17="X",60*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="H17" s="16" t="str">
+        <f>IF($C17=ML,"X","")</f>
+        <v/>
+      </c>
+      <c r="I17" s="16" t="str">
+        <f>IF(H17="X",30*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="J17" s="16" t="str">
+        <f>IF($C17=NL,"X","")</f>
+        <v/>
+      </c>
+      <c r="K17" s="16" t="str">
+        <f t="shared" ref="K17:K19" si="4">IF($J17="X",0,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18" spans="1:11" ht="36" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="A18" s="70"/>
+      <c r="B18" s="30" t="str">
+        <f>RUBRICA!A10</f>
+        <v>7. Entrega la documentación y evidencias requerida por la asignatura de acuerdo a la estrucutra y nombres solicitados, guardando todas las evidencias de avances en Git</v>
+      </c>
+      <c r="C18" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="D18" s="16"/>
+      <c r="E18" s="16" t="str">
+        <f>IF(D18="X",100*0.15,"")</f>
+        <v/>
+      </c>
+      <c r="F18" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="G18" s="16">
+        <f>IF(F18="X",60*0.15,"")</f>
+        <v>9</v>
+      </c>
+      <c r="H18" s="16" t="str">
+        <f>IF($C18=ML,"X","")</f>
+        <v/>
+      </c>
+      <c r="I18" s="16" t="str">
+        <f>IF(H18="X",30*0.15,"")</f>
+        <v/>
+      </c>
+      <c r="J18" s="16" t="str">
+        <f>IF($C18=NL,"X","")</f>
+        <v/>
+      </c>
+      <c r="K18" s="16" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:11" ht="48" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="42"/>
-      <c r="B15" s="28" t="str">
-        <f>RUBRICA!A6</f>
-        <v>3. Genera evidencias que dan cuenta del avance del Proyecto APT en relación a documentación, programación y almacenamiento de datos , de acuerdo a lo planificado por el equipo y que cumpla con estándares de desarrollo de la industria</v>
-      </c>
-      <c r="C15" s="26" t="s">
-        <v>5</v>
-      </c>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15" t="str">
-        <f>IF(D15="X",100*0.25,"")</f>
+    <row r="19" spans="1:11" ht="22.9" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.25">
+      <c r="A19" s="70"/>
+      <c r="B19" s="30" t="str">
+        <f>RUBRICA!A12</f>
+        <v>9.-Generan evidencias claras dentro del repositorio  del aporte de cada uno de los integrantes del equipo que permitan identificar la equidad en el trabajo y la participación de cada estudiante.</v>
+      </c>
+      <c r="C19" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="D19" s="16" t="str">
+        <f>IF($C19=CL,"X","")</f>
+        <v>X</v>
+      </c>
+      <c r="E19" s="16">
+        <f>IF(D19="X",100*0.15,"")</f>
+        <v>15</v>
+      </c>
+      <c r="F19" s="16" t="str">
+        <f>IF($C19=L,"X","")</f>
         <v/>
       </c>
-      <c r="F15" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="G15" s="15">
-        <f>IF(F15="X",60*0.25,"")</f>
-        <v>15</v>
-      </c>
-      <c r="H15" s="15" t="str">
-        <f t="shared" si="2"/>
+      <c r="G19" s="16" t="str">
+        <f>IF(F19="X",60*0.15,"")</f>
         <v/>
       </c>
-      <c r="I15" s="15" t="str">
-        <f>IF(H15="X",30*0.25,"")</f>
+      <c r="H19" s="16" t="str">
+        <f>IF($C19=ML,"X","")</f>
         <v/>
       </c>
-      <c r="J15" s="15" t="str">
-        <f t="shared" si="3"/>
+      <c r="I19" s="16" t="str">
+        <f>IF(H19="X",30*0.15,"")</f>
         <v/>
       </c>
-      <c r="K15" s="15" t="str">
+      <c r="J19" s="16" t="str">
+        <f>IF($C19=NL,"X","")</f>
+        <v/>
+      </c>
+      <c r="K19" s="16" t="str">
         <f t="shared" si="4"/>
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:11" ht="24" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A16" s="42"/>
-      <c r="B16" s="28" t="str">
-        <f>RUBRICA!A7</f>
-        <v>4. Utiliza de manera precisa el lenguaje técnico en los entregables de acuerdo con lo requerido por la disciplina.</v>
-      </c>
-      <c r="C16" s="26" t="s">
+    <row r="20" spans="1:11" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A20" s="67"/>
+      <c r="B20" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="C20" s="33">
+        <f>E20+G20+I20+K20</f>
+        <v>53</v>
+      </c>
+      <c r="D20" s="19"/>
+      <c r="E20" s="19">
+        <f>SUM(E13:E19)</f>
+        <v>20</v>
+      </c>
+      <c r="F20" s="19"/>
+      <c r="G20" s="19">
+        <f>SUM(G13:G19)</f>
+        <v>33</v>
+      </c>
+      <c r="H20" s="19"/>
+      <c r="I20" s="19">
+        <f>SUM(I13:I19)</f>
+        <v>0</v>
+      </c>
+      <c r="J20" s="19"/>
+      <c r="K20" s="19">
+        <f>SUM(K13:K19)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:11" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
+      <c r="A21" s="54"/>
+      <c r="B21" s="32" t="s">
+        <v>67</v>
+      </c>
+      <c r="C21" s="20">
+        <f>VLOOKUP(C20,ESCALA_IEP!A1:B152,2,FALSE)</f>
+        <v>4.8</v>
+      </c>
+    </row>
+    <row r="22" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="24" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A24" s="66" t="s">
+        <v>59</v>
+      </c>
+      <c r="B24" s="53" t="s">
+        <v>68</v>
+      </c>
+      <c r="C24" s="55" t="str">
+        <f>$B$4</f>
+        <v>Esteban Fierro</v>
+      </c>
+      <c r="D24" s="56"/>
+      <c r="E24" s="56"/>
+      <c r="F24" s="56"/>
+      <c r="G24" s="56"/>
+      <c r="H24" s="56"/>
+      <c r="I24" s="56"/>
+      <c r="J24" s="56"/>
+      <c r="K24" s="57"/>
+    </row>
+    <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A25" s="67"/>
+      <c r="B25" s="54"/>
+      <c r="C25" s="58"/>
+      <c r="D25" s="59"/>
+      <c r="E25" s="59"/>
+      <c r="F25" s="59"/>
+      <c r="G25" s="59"/>
+      <c r="H25" s="59"/>
+      <c r="I25" s="59"/>
+      <c r="J25" s="59"/>
+      <c r="K25" s="60"/>
+    </row>
+    <row r="26" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="67"/>
+      <c r="B26" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="C26" s="61" t="s">
+        <v>60</v>
+      </c>
+      <c r="D26" s="62" t="s">
+        <v>61</v>
+      </c>
+      <c r="E26" s="63"/>
+      <c r="F26" s="63"/>
+      <c r="G26" s="63"/>
+      <c r="H26" s="63"/>
+      <c r="I26" s="63"/>
+      <c r="J26" s="63"/>
+      <c r="K26" s="64"/>
+    </row>
+    <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="67"/>
+      <c r="B27" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C27" s="54"/>
+      <c r="D27" s="62" t="s">
+        <v>63</v>
+      </c>
+      <c r="E27" s="64"/>
+      <c r="F27" s="62" t="s">
+        <v>64</v>
+      </c>
+      <c r="G27" s="64"/>
+      <c r="H27" s="65" t="s">
+        <v>65</v>
+      </c>
+      <c r="I27" s="64"/>
+      <c r="J27" s="62" t="s">
+        <v>6</v>
+      </c>
+      <c r="K27" s="64"/>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" s="67"/>
+      <c r="B28" s="30" t="str">
+        <f>RUBRICA!A6</f>
+        <v>3. Relaciona el Proyecto APT con sus intereses profesionales. *</v>
+      </c>
+      <c r="C28" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="D28" s="16" t="str">
+        <f t="shared" ref="D28:D30" si="5">IF($C28=CL,"X","")</f>
+        <v>X</v>
+      </c>
+      <c r="E28" s="16">
+        <f>IF(D28="X",100*0.05,"")</f>
         <v>5</v>
       </c>
-      <c r="D16" s="15" t="str">
-        <f t="shared" si="0"/>
+      <c r="F28" s="16" t="str">
+        <f t="shared" ref="F28:F30" si="6">IF($C28=L,"X","")</f>
+        <v/>
+      </c>
+      <c r="G28" s="16" t="str">
+        <f>IF(F28="X",60*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="H28" s="16" t="str">
+        <f t="shared" ref="H28:H30" si="7">IF($C28=ML,"X","")</f>
+        <v/>
+      </c>
+      <c r="I28" s="16" t="str">
+        <f>IF(H28="X",30*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="J28" s="16" t="str">
+        <f t="shared" ref="J28:J30" si="8">IF($C28=NL,"X","")</f>
+        <v/>
+      </c>
+      <c r="K28" s="16" t="str">
+        <f t="shared" ref="K28:K30" si="9">IF($J28="X",0,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29" spans="1:11" ht="24.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="67"/>
+      <c r="B29" s="30" t="str">
+        <f>RUBRICA!A11</f>
+        <v>8. Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información. *</v>
+      </c>
+      <c r="C29" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="D29" s="16"/>
+      <c r="E29" s="16" t="str">
+        <f>IF(D29="X",100*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="F29" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="G29" s="16">
+        <f>IF(F29="X",60*0.1,"")</f>
+        <v>6</v>
+      </c>
+      <c r="H29" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="I29" s="16" t="str">
+        <f>IF(H29="X",30*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="J29" s="16" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="K29" s="16" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="1:11" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="67"/>
+      <c r="B30" s="30" t="str">
+        <f>RUBRICA!A13</f>
+        <v>10. Colaboración y trabajo en equipo *</v>
+      </c>
+      <c r="C30" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="D30" s="16" t="str">
+        <f t="shared" si="5"/>
         <v>X</v>
       </c>
-      <c r="E16" s="15">
-        <f>IF(D16="X",100*0.05,"")</f>
+      <c r="E30" s="16">
+        <f>IF(D30="X",100*0.1,"")</f>
+        <v>10</v>
+      </c>
+      <c r="F30" s="16" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+      <c r="G30" s="16" t="str">
+        <f>IF(F30="X",60*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="H30" s="16" t="str">
+        <f t="shared" si="7"/>
+        <v/>
+      </c>
+      <c r="I30" s="16" t="str">
+        <f>IF(H30="X",30*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="J30" s="16" t="str">
+        <f t="shared" si="8"/>
+        <v/>
+      </c>
+      <c r="K30" s="16" t="str">
+        <f t="shared" si="9"/>
+        <v/>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A31" s="67"/>
+      <c r="B31" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="C31" s="18">
+        <f>E31+G31+I31+K31</f>
+        <v>21</v>
+      </c>
+      <c r="D31" s="19"/>
+      <c r="E31" s="19">
+        <f>SUM(E28:E30)</f>
+        <v>15</v>
+      </c>
+      <c r="F31" s="19"/>
+      <c r="G31" s="19">
+        <f>SUM(G28:G30)</f>
+        <v>6</v>
+      </c>
+      <c r="H31" s="19"/>
+      <c r="I31" s="19">
+        <f>SUM(I28:I30)</f>
+        <v>0</v>
+      </c>
+      <c r="J31" s="19"/>
+      <c r="K31" s="19">
+        <f>SUM(K29:K30)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A32" s="54"/>
+      <c r="B32" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="C32" s="20">
+        <f>VLOOKUP(C31,ESCALA_TRAB_EQUIP!A1:B52,2,FALSE)</f>
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="33" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="22"/>
+      <c r="C33" s="23"/>
+    </row>
+    <row r="34" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="22"/>
+      <c r="C34" s="23"/>
+    </row>
+    <row r="35" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="36" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A36" s="66" t="s">
+        <v>59</v>
+      </c>
+      <c r="B36" s="53" t="s">
+        <v>68</v>
+      </c>
+      <c r="C36" s="55" t="str">
+        <f>B5</f>
+        <v>Francisca Herrera</v>
+      </c>
+      <c r="D36" s="56"/>
+      <c r="E36" s="56"/>
+      <c r="F36" s="56"/>
+      <c r="G36" s="56"/>
+      <c r="H36" s="56"/>
+      <c r="I36" s="56"/>
+      <c r="J36" s="56"/>
+      <c r="K36" s="57"/>
+    </row>
+    <row r="37" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="67"/>
+      <c r="B37" s="54"/>
+      <c r="C37" s="58"/>
+      <c r="D37" s="59"/>
+      <c r="E37" s="59"/>
+      <c r="F37" s="59"/>
+      <c r="G37" s="59"/>
+      <c r="H37" s="59"/>
+      <c r="I37" s="59"/>
+      <c r="J37" s="59"/>
+      <c r="K37" s="60"/>
+    </row>
+    <row r="38" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="67"/>
+      <c r="B38" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="C38" s="61" t="s">
+        <v>60</v>
+      </c>
+      <c r="D38" s="62" t="s">
+        <v>61</v>
+      </c>
+      <c r="E38" s="63"/>
+      <c r="F38" s="63"/>
+      <c r="G38" s="63"/>
+      <c r="H38" s="63"/>
+      <c r="I38" s="63"/>
+      <c r="J38" s="63"/>
+      <c r="K38" s="64"/>
+    </row>
+    <row r="39" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="67"/>
+      <c r="B39" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C39" s="54"/>
+      <c r="D39" s="62" t="s">
+        <v>63</v>
+      </c>
+      <c r="E39" s="64"/>
+      <c r="F39" s="62" t="s">
+        <v>64</v>
+      </c>
+      <c r="G39" s="64"/>
+      <c r="H39" s="65" t="s">
+        <v>65</v>
+      </c>
+      <c r="I39" s="64"/>
+      <c r="J39" s="62" t="s">
+        <v>6</v>
+      </c>
+      <c r="K39" s="64"/>
+    </row>
+    <row r="40" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="67"/>
+      <c r="B40" s="30" t="str">
+        <f>RUBRICA!A6</f>
+        <v>3. Relaciona el Proyecto APT con sus intereses profesionales. *</v>
+      </c>
+      <c r="C40" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="D40" s="16" t="str">
+        <f t="shared" ref="D40:D42" si="10">IF($C40=CL,"X","")</f>
+        <v>X</v>
+      </c>
+      <c r="E40" s="16">
+        <f>IF(D40="X",100*0.05,"")</f>
         <v>5</v>
       </c>
-      <c r="F16" s="15" t="str">
-        <f t="shared" si="1"/>
+      <c r="F40" s="16" t="str">
+        <f t="shared" ref="F40:F42" si="11">IF($C40=L,"X","")</f>
         <v/>
       </c>
-      <c r="G16" s="15" t="str">
-        <f>IF(F16="X",60*0.05,"")</f>
+      <c r="G40" s="16" t="str">
+        <f>IF(F40="X",60*0.05,"")</f>
         <v/>
       </c>
-      <c r="H16" s="15" t="str">
-        <f t="shared" si="2"/>
+      <c r="H40" s="16" t="str">
+        <f t="shared" ref="H40:H42" si="12">IF($C40=ML,"X","")</f>
         <v/>
       </c>
-      <c r="I16" s="15" t="str">
-        <f>IF(H16="X",30*0.05,"")</f>
+      <c r="I40" s="16" t="str">
+        <f>IF(H40="X",30*0.05,"")</f>
         <v/>
       </c>
-      <c r="J16" s="15" t="str">
-        <f t="shared" si="3"/>
+      <c r="J40" s="16" t="str">
+        <f t="shared" ref="J40:J42" si="13">IF($C40=NL,"X","")</f>
         <v/>
       </c>
-      <c r="K16" s="15" t="str">
-        <f t="shared" si="4"/>
+      <c r="K40" s="16" t="str">
+        <f t="shared" ref="K40:K42" si="14">IF($J40="X",0,"")</f>
         <v/>
       </c>
     </row>
-    <row r="17" spans="1:11" ht="24" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="42"/>
-      <c r="B17" s="28" t="str">
-        <f>RUBRICA!A8</f>
-        <v xml:space="preserve">5. Utiliza reglas de redacción, ortografía (literal, puntual, acentual) y las normas para citas y referencias. </v>
-      </c>
-      <c r="C17" s="26" t="s">
+    <row r="41" spans="1:11" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A41" s="67"/>
+      <c r="B41" s="30" t="str">
+        <f>RUBRICA!A11</f>
+        <v>8. Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información. *</v>
+      </c>
+      <c r="C41" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="D41" s="16"/>
+      <c r="E41" s="16" t="str">
+        <f>IF(D41="X",100*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="F41" s="16" t="s">
+        <v>78</v>
+      </c>
+      <c r="G41" s="16">
+        <f>IF(F41="X",60*0.1,"")</f>
+        <v>6</v>
+      </c>
+      <c r="H41" s="16" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="I41" s="16" t="str">
+        <f>IF(H41="X",30*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="J41" s="16" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="K41" s="16" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
+    </row>
+    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A42" s="67"/>
+      <c r="B42" s="30" t="str">
+        <f>RUBRICA!A13</f>
+        <v>10. Colaboración y trabajo en equipo *</v>
+      </c>
+      <c r="C42" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="D42" s="16" t="str">
+        <f t="shared" si="10"/>
+        <v>X</v>
+      </c>
+      <c r="E42" s="16">
+        <f>IF(D42="X",100*0.1,"")</f>
+        <v>10</v>
+      </c>
+      <c r="F42" s="16" t="str">
+        <f t="shared" si="11"/>
+        <v/>
+      </c>
+      <c r="G42" s="16" t="str">
+        <f>IF(F42="X",60*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="H42" s="16" t="str">
+        <f t="shared" si="12"/>
+        <v/>
+      </c>
+      <c r="I42" s="16" t="str">
+        <f>IF(H42="X",30*0.1,"")</f>
+        <v/>
+      </c>
+      <c r="J42" s="16" t="str">
+        <f t="shared" si="13"/>
+        <v/>
+      </c>
+      <c r="K42" s="16" t="str">
+        <f t="shared" si="14"/>
+        <v/>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A43" s="67"/>
+      <c r="B43" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="C43" s="18">
+        <f>E43+G43+I43+K43</f>
+        <v>21</v>
+      </c>
+      <c r="D43" s="19"/>
+      <c r="E43" s="19">
+        <f>SUM(E40:E42)</f>
+        <v>15</v>
+      </c>
+      <c r="F43" s="19"/>
+      <c r="G43" s="19">
+        <f>SUM(G40:G42)</f>
+        <v>6</v>
+      </c>
+      <c r="H43" s="19"/>
+      <c r="I43" s="19">
+        <f>SUM(I40:I42)</f>
+        <v>0</v>
+      </c>
+      <c r="J43" s="19"/>
+      <c r="K43" s="19">
+        <f>SUM(K41:K42)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A44" s="54"/>
+      <c r="B44" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="C44" s="20">
+        <f>VLOOKUP(C43,ESCALA_TRAB_EQUIP!A1:B52,2,FALSE)</f>
+        <v>5.8</v>
+      </c>
+    </row>
+    <row r="45" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B45" s="22"/>
+      <c r="C45" s="23"/>
+    </row>
+    <row r="46" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B46" s="22"/>
+      <c r="C46" s="23"/>
+    </row>
+    <row r="47" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="66" t="s">
+        <v>59</v>
+      </c>
+      <c r="B47" s="53" t="s">
+        <v>68</v>
+      </c>
+      <c r="C47" s="55">
+        <f>B6</f>
+        <v>0</v>
+      </c>
+      <c r="D47" s="56"/>
+      <c r="E47" s="56"/>
+      <c r="F47" s="56"/>
+      <c r="G47" s="56"/>
+      <c r="H47" s="56"/>
+      <c r="I47" s="56"/>
+      <c r="J47" s="56"/>
+      <c r="K47" s="57"/>
+    </row>
+    <row r="48" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="67"/>
+      <c r="B48" s="54"/>
+      <c r="C48" s="58"/>
+      <c r="D48" s="59"/>
+      <c r="E48" s="59"/>
+      <c r="F48" s="59"/>
+      <c r="G48" s="59"/>
+      <c r="H48" s="59"/>
+      <c r="I48" s="59"/>
+      <c r="J48" s="59"/>
+      <c r="K48" s="60"/>
+    </row>
+    <row r="49" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A49" s="67"/>
+      <c r="B49" s="14" t="s">
+        <v>69</v>
+      </c>
+      <c r="C49" s="61" t="s">
+        <v>60</v>
+      </c>
+      <c r="D49" s="62" t="s">
+        <v>61</v>
+      </c>
+      <c r="E49" s="63"/>
+      <c r="F49" s="63"/>
+      <c r="G49" s="63"/>
+      <c r="H49" s="63"/>
+      <c r="I49" s="63"/>
+      <c r="J49" s="63"/>
+      <c r="K49" s="64"/>
+    </row>
+    <row r="50" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A50" s="67"/>
+      <c r="B50" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="C50" s="54"/>
+      <c r="D50" s="62" t="s">
+        <v>63</v>
+      </c>
+      <c r="E50" s="64"/>
+      <c r="F50" s="62" t="s">
+        <v>64</v>
+      </c>
+      <c r="G50" s="64"/>
+      <c r="H50" s="65" t="s">
+        <v>65</v>
+      </c>
+      <c r="I50" s="64"/>
+      <c r="J50" s="62" t="s">
+        <v>6</v>
+      </c>
+      <c r="K50" s="64"/>
+    </row>
+    <row r="51" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A51" s="67"/>
+      <c r="B51" s="30" t="str">
+        <f>RUBRICA!A6</f>
+        <v>3. Relaciona el Proyecto APT con sus intereses profesionales. *</v>
+      </c>
+      <c r="C51" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="D51" s="16" t="str">
+        <f t="shared" ref="D51:D53" si="15">IF($C51=CL,"X","")</f>
+        <v>X</v>
+      </c>
+      <c r="E51" s="16">
+        <f>IF(D51="X",100*0.05,"")</f>
         <v>5</v>
       </c>
-      <c r="D17" s="15" t="str">
-        <f t="shared" si="0"/>
+      <c r="F51" s="16" t="str">
+        <f t="shared" ref="F51:F53" si="16">IF($C51=L,"X","")</f>
+        <v/>
+      </c>
+      <c r="G51" s="16" t="str">
+        <f>IF(F51="X",60*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="H51" s="16" t="str">
+        <f t="shared" ref="H51:H53" si="17">IF($C51=ML,"X","")</f>
+        <v/>
+      </c>
+      <c r="I51" s="16" t="str">
+        <f>IF(H51="X",30*0.05,"")</f>
+        <v/>
+      </c>
+      <c r="J51" s="16" t="str">
+        <f t="shared" ref="J51:J53" si="18">IF($C51=NL,"X","")</f>
+        <v/>
+      </c>
+      <c r="K51" s="16" t="str">
+        <f t="shared" ref="K51:K53" si="19">IF($J51="X",0,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52" spans="1:11" ht="25.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="67"/>
+      <c r="B52" s="30" t="str">
+        <f>RUBRICA!A11</f>
+        <v>8. Expone el tema utilizando un lenguaje técnico disciplinar al presentar la propuesta y responde evidenciando un manejo de la información. *</v>
+      </c>
+      <c r="C52" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="D52" s="16" t="str">
+        <f t="shared" si="15"/>
         <v>X</v>
       </c>
-      <c r="E17" s="15">
-        <f>IF(D17="X",100*0.05,"")</f>
-        <v>5</v>
-      </c>
-      <c r="F17" s="15" t="str">
-        <f t="shared" si="1"/>
+      <c r="E52" s="16">
+        <f>IF(D52="X",100*0.1,"")</f>
+        <v>10</v>
+      </c>
+      <c r="F52" s="16" t="str">
+        <f t="shared" si="16"/>
         <v/>
       </c>
-      <c r="G17" s="15" t="str">
-        <f>IF(F17="X",60*0.05,"")</f>
+      <c r="G52" s="16" t="str">
+        <f>IF(F52="X",60*0.1,"")</f>
         <v/>
       </c>
-      <c r="H17" s="15" t="str">
-        <f t="shared" si="2"/>
+      <c r="H52" s="16" t="str">
+        <f t="shared" si="17"/>
         <v/>
       </c>
-      <c r="I17" s="15" t="str">
-        <f>IF(H17="X",30*0.05,"")</f>
+      <c r="I52" s="16" t="str">
+        <f>IF(H52="X",30*0.1,"")</f>
         <v/>
       </c>
-      <c r="J17" s="15" t="str">
-        <f t="shared" si="3"/>
+      <c r="J52" s="16" t="str">
+        <f t="shared" si="18"/>
         <v/>
       </c>
-      <c r="K17" s="15" t="str">
-        <f t="shared" si="4"/>
+      <c r="K52" s="16" t="str">
+        <f t="shared" si="19"/>
         <v/>
       </c>
     </row>
-    <row r="18" spans="1:11" ht="36" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="42"/>
-      <c r="B18" s="28" t="str">
-        <f>RUBRICA!A9</f>
-        <v>6. Entrega la documentación y evidencias requerida por la asignatura de acuerdo a la estrucutra y nombres solicitados, guardando todas las evidencias de avances en Git</v>
-      </c>
-      <c r="C18" s="26" t="s">
-        <v>5</v>
-      </c>
-      <c r="D18" s="15" t="str">
-        <f>IF($C18=CL,"X","")</f>
+    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A53" s="67"/>
+      <c r="B53" s="30" t="str">
+        <f>RUBRICA!A13</f>
+        <v>10. Colaboración y trabajo en equipo *</v>
+      </c>
+      <c r="C53" s="28" t="s">
+        <v>63</v>
+      </c>
+      <c r="D53" s="16" t="str">
+        <f t="shared" si="15"/>
         <v>X</v>
       </c>
-      <c r="E18" s="15">
-        <f>IF(D18="X",100*0.2,"")</f>
-        <v>20</v>
-      </c>
-      <c r="F18" s="15" t="str">
-        <f>IF($C18=L,"X","")</f>
+      <c r="E53" s="16">
+        <f>IF(D53="X",100*0.1,"")</f>
+        <v>10</v>
+      </c>
+      <c r="F53" s="16" t="str">
+        <f t="shared" si="16"/>
         <v/>
       </c>
-      <c r="G18" s="15" t="str">
-        <f>IF(F18="X",60*0.2,"")</f>
+      <c r="G53" s="16" t="str">
+        <f>IF(F53="X",60*0.1,"")</f>
         <v/>
       </c>
-      <c r="H18" s="15" t="str">
-        <f>IF($C18=ML,"X","")</f>
+      <c r="H53" s="16" t="str">
+        <f t="shared" si="17"/>
         <v/>
       </c>
-      <c r="I18" s="15" t="str">
-        <f>IF(H18="X",30*0.2,"")</f>
+      <c r="I53" s="16" t="str">
+        <f>IF(H53="X",30*0.1,"")</f>
         <v/>
       </c>
-      <c r="J18" s="15" t="str">
-        <f>IF($C18=NL,"X","")</f>
+      <c r="J53" s="16" t="str">
+        <f t="shared" si="18"/>
         <v/>
       </c>
-      <c r="K18" s="15" t="str">
-        <f t="shared" ref="K18:K20" si="5">IF($J18="X",0,"")</f>
+      <c r="K53" s="16" t="str">
+        <f t="shared" si="19"/>
         <v/>
       </c>
     </row>
-    <row r="19" spans="1:11" ht="36" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="42"/>
-      <c r="B19" s="28" t="str">
-        <f>RUBRICA!A10</f>
-        <v>7.- Generan evidencias claras dentro del repositorio  del aporte de cada uno de los integrantes del equipo que permitan identificar la equidad en el trabajo y la participación de cada estudiante.</v>
-      </c>
-      <c r="C19" s="26" t="s">
-        <v>5</v>
-      </c>
-      <c r="D19" s="15" t="str">
-        <f>IF($C19=CL,"X","")</f>
-        <v>X</v>
-      </c>
-      <c r="E19" s="15">
-        <f>IF(D19="X",100*0.15,"")</f>
-        <v>15</v>
-      </c>
-      <c r="F19" s="15" t="str">
-        <f>IF($C19=L,"X","")</f>
-        <v/>
-      </c>
-      <c r="G19" s="15" t="str">
-        <f>IF(F19="X",60*0.15,"")</f>
-        <v/>
-      </c>
-      <c r="H19" s="15" t="str">
-        <f>IF($C19=ML,"X","")</f>
-        <v/>
-      </c>
-      <c r="I19" s="15" t="str">
-        <f>IF(H19="X",30*0.15,"")</f>
-        <v/>
-      </c>
-      <c r="J19" s="15" t="str">
-        <f>IF($C19=NL,"X","")</f>
-        <v/>
-      </c>
-      <c r="K19" s="15" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-    </row>
-    <row r="20" spans="1:11" ht="36" outlineLevel="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="42"/>
-      <c r="B20" s="28" t="str">
-        <f>RUBRICA!A11</f>
-        <v>8. Demuestra un trabajo en equipo en donde todos los miembros del equipo expresan con fluidez el conocimiento del tema expuesto y  participan de las actividades planificadas en el proyecto</v>
-      </c>
-      <c r="C20" s="26" t="s">
-        <v>5</v>
-      </c>
-      <c r="D20" s="15" t="str">
-        <f>IF($C20=CL,"X","")</f>
-        <v>X</v>
-      </c>
-      <c r="E20" s="15">
-        <f>IF(D20="X",100*0.1,"")</f>
-        <v>10</v>
-      </c>
-      <c r="F20" s="15" t="str">
-        <f>IF($C20=L,"X","")</f>
-        <v/>
-      </c>
-      <c r="G20" s="15" t="str">
-        <f>IF(F20="X",60*0.1,"")</f>
-        <v/>
-      </c>
-      <c r="H20" s="15" t="str">
-        <f>IF($C20=ML,"X","")</f>
-        <v/>
-      </c>
-      <c r="I20" s="15" t="str">
-        <f>IF(H20="X",30*0.1,"")</f>
-        <v/>
-      </c>
-      <c r="J20" s="15" t="str">
-        <f>IF($C20=NL,"X","")</f>
-        <v/>
-      </c>
-      <c r="K20" s="15" t="str">
-        <f t="shared" si="5"/>
-        <v/>
-      </c>
-    </row>
-    <row r="21" spans="1:11" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="41"/>
-      <c r="B21" s="27" t="s">
-        <v>4</v>
-      </c>
-      <c r="C21" s="31">
-        <f>E21+G21+I21+K21</f>
-        <v>90</v>
-      </c>
-      <c r="D21" s="16"/>
-      <c r="E21" s="16">
-        <f>SUM(E13:E20)</f>
-        <v>75</v>
-      </c>
-      <c r="F21" s="16"/>
-      <c r="G21" s="16">
-        <f>SUM(G13:G20)</f>
-        <v>15</v>
-      </c>
-      <c r="H21" s="16"/>
-      <c r="I21" s="16">
-        <f>SUM(I13:I20)</f>
+    <row r="54" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A54" s="67"/>
+      <c r="B54" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="C54" s="18">
+        <f>E54+G54+I54+K54</f>
+        <v>25</v>
+      </c>
+      <c r="D54" s="19"/>
+      <c r="E54" s="19">
+        <f>SUM(E51:E53)</f>
+        <v>25</v>
+      </c>
+      <c r="F54" s="19"/>
+      <c r="G54" s="19">
+        <f>SUM(G51:G53)</f>
         <v>0</v>
       </c>
-      <c r="J21" s="16"/>
-      <c r="K21" s="16">
-        <f>SUM(K13:K20)</f>
+      <c r="H54" s="19"/>
+      <c r="I54" s="19">
+        <f>SUM(I51:I53)</f>
         <v>0</v>
       </c>
-    </row>
-    <row r="22" spans="1:11" ht="15.75" customHeight="1" outlineLevel="1" x14ac:dyDescent="0.3">
-      <c r="A22" s="43"/>
-      <c r="B22" s="30" t="s">
-        <v>13</v>
-      </c>
-      <c r="C22" s="17">
-        <f>VLOOKUP(C21,ESCALA_IEP!A2:B202,2,FALSE)</f>
-        <v>6.3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D23" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="24" spans="1:11" ht="48" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B24" s="34"/>
-    </row>
-    <row r="25" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="18"/>
-      <c r="C25" s="19"/>
-    </row>
-    <row r="26" spans="1:11" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="35"/>
-    </row>
-    <row r="27" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="28" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="29" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="30" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="31" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="32" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="33" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="34" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="35" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="36" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="37" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="38" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="39" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="40" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="41" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="43" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="44" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="45" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="46" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="47" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="48" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="49" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="50" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="51" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="52" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="53" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="54" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="55" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="56" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="57" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="58" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="59" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="60" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="61" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="62" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="63" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="64" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+      <c r="J54" s="19"/>
+      <c r="K54" s="19">
+        <f>SUM(K52:K53)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="54"/>
+      <c r="B55" s="17" t="s">
+        <v>67</v>
+      </c>
+      <c r="C55" s="20">
+        <f>VLOOKUP(C54,ESCALA_TRAB_EQUIP!A1:B52,2,FALSE)</f>
+        <v>7</v>
+      </c>
+    </row>
+    <row r="56" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B56" s="22"/>
+      <c r="C56" s="23"/>
+    </row>
+    <row r="57" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="58" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="59" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="60" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="61" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="62" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="63" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="64" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="65" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="66" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="67" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2614,17 +3617,76 @@
     <row r="893" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="894" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="895" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="896" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="897" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="898" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="899" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="900" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="901" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="902" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="903" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="904" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="905" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="906" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="907" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="908" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="909" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="910" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="911" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="912" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="913" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="914" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="915" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="916" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="917" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="918" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="919" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="920" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="921" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="922" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="923" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="924" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="925" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="926" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="7">
-    <mergeCell ref="A11:A22"/>
+  <mergeCells count="35">
+    <mergeCell ref="B47:B48"/>
+    <mergeCell ref="C49:C50"/>
+    <mergeCell ref="C47:K48"/>
+    <mergeCell ref="J50:K50"/>
+    <mergeCell ref="A47:A55"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="D49:K49"/>
+    <mergeCell ref="D50:E50"/>
+    <mergeCell ref="F50:G50"/>
+    <mergeCell ref="H50:I50"/>
+    <mergeCell ref="A36:A44"/>
+    <mergeCell ref="A24:A32"/>
+    <mergeCell ref="E2:E3"/>
     <mergeCell ref="C11:C12"/>
     <mergeCell ref="D12:E12"/>
     <mergeCell ref="D11:K11"/>
     <mergeCell ref="F12:G12"/>
     <mergeCell ref="H12:I12"/>
     <mergeCell ref="J12:K12"/>
+    <mergeCell ref="A11:A21"/>
+    <mergeCell ref="B24:B25"/>
+    <mergeCell ref="C24:K25"/>
+    <mergeCell ref="C26:C27"/>
+    <mergeCell ref="D26:K26"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="B36:B37"/>
+    <mergeCell ref="C36:K37"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="D38:K38"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="F39:G39"/>
+    <mergeCell ref="H39:I39"/>
+    <mergeCell ref="J39:K39"/>
   </mergeCells>
-  <conditionalFormatting sqref="C4:C6">
+  <conditionalFormatting sqref="C4:E6">
     <cfRule type="cellIs" dxfId="1" priority="1" operator="lessThan">
       <formula>4</formula>
     </cfRule>
@@ -2633,7 +3695,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Error de Ingreso - Nota debe estar entre 1,0 y 7,0" sqref="C4:C6" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="decimal" allowBlank="1" showInputMessage="1" showErrorMessage="1" prompt="Error de Ingreso - Nota debe estar entre 1,0 y 7,0" sqref="C4:E6" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>1</formula1>
       <formula2>7</formula2>
     </dataValidation>
@@ -2647,233 +3709,11 @@
           <x14:formula1>
             <xm:f>'RELEVANCIA-PUNTAJE'!$B$2:$E$2</xm:f>
           </x14:formula1>
-          <xm:sqref>C13:C20</xm:sqref>
+          <xm:sqref>C40:C42 C13:C19 C28:C30 C51:C53</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
   </extLst>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8B396D1B-8A63-4A90-BA20-D34AC13A3962}">
-  <dimension ref="A1:F11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="6" width="38.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="49" t="s">
-        <v>14</v>
-      </c>
-      <c r="B1" s="51" t="s">
-        <v>15</v>
-      </c>
-      <c r="C1" s="52"/>
-      <c r="D1" s="52"/>
-      <c r="E1" s="53"/>
-      <c r="F1" s="49" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
-      <c r="A2" s="50"/>
-      <c r="B2" s="55" t="s">
-        <v>25</v>
-      </c>
-      <c r="C2" s="55" t="s">
-        <v>17</v>
-      </c>
-      <c r="D2" s="21" t="s">
-        <v>18</v>
-      </c>
-      <c r="E2" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" s="50"/>
-    </row>
-    <row r="3" spans="1:6" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="50"/>
-      <c r="B3" s="56"/>
-      <c r="C3" s="56"/>
-      <c r="D3" s="37">
-        <v>-0.3</v>
-      </c>
-      <c r="E3" s="37">
-        <v>0</v>
-      </c>
-      <c r="F3" s="54"/>
-    </row>
-    <row r="4" spans="1:6" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="24" t="s">
-        <v>26</v>
-      </c>
-      <c r="B4" s="24" t="s">
-        <v>27</v>
-      </c>
-      <c r="C4" s="24" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" s="24" t="s">
-        <v>29</v>
-      </c>
-      <c r="E4" s="24" t="s">
-        <v>30</v>
-      </c>
-      <c r="F4" s="23">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="24" t="s">
-        <v>31</v>
-      </c>
-      <c r="B5" s="24" t="s">
-        <v>42</v>
-      </c>
-      <c r="C5" s="24" t="s">
-        <v>32</v>
-      </c>
-      <c r="D5" s="24" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" s="24" t="s">
-        <v>34</v>
-      </c>
-      <c r="F5" s="23">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="90" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="24" t="s">
-        <v>43</v>
-      </c>
-      <c r="B6" s="24" t="s">
-        <v>44</v>
-      </c>
-      <c r="C6" s="24" t="s">
-        <v>45</v>
-      </c>
-      <c r="D6" s="24" t="s">
-        <v>46</v>
-      </c>
-      <c r="E6" s="24" t="s">
-        <v>47</v>
-      </c>
-      <c r="F6" s="23">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="39" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="24" t="s">
-        <v>48</v>
-      </c>
-      <c r="B7" s="24" t="s">
-        <v>49</v>
-      </c>
-      <c r="C7" s="24" t="s">
-        <v>50</v>
-      </c>
-      <c r="D7" s="24" t="s">
-        <v>51</v>
-      </c>
-      <c r="E7" s="24" t="s">
-        <v>52</v>
-      </c>
-      <c r="F7" s="23">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="51" x14ac:dyDescent="0.25">
-      <c r="A8" s="24" t="s">
-        <v>35</v>
-      </c>
-      <c r="B8" s="24" t="s">
-        <v>22</v>
-      </c>
-      <c r="C8" s="24" t="s">
-        <v>19</v>
-      </c>
-      <c r="D8" s="24" t="s">
-        <v>20</v>
-      </c>
-      <c r="E8" s="24" t="s">
-        <v>21</v>
-      </c>
-      <c r="F8" s="38">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="51.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="24" t="s">
-        <v>53</v>
-      </c>
-      <c r="B9" s="24" t="s">
-        <v>54</v>
-      </c>
-      <c r="C9" s="24" t="s">
-        <v>55</v>
-      </c>
-      <c r="D9" s="24" t="s">
-        <v>56</v>
-      </c>
-      <c r="E9" s="24" t="s">
-        <v>57</v>
-      </c>
-      <c r="F9" s="23">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="64.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="39" t="s">
-        <v>58</v>
-      </c>
-      <c r="B10" s="39" t="s">
-        <v>59</v>
-      </c>
-      <c r="C10" s="39" t="s">
-        <v>60</v>
-      </c>
-      <c r="D10" s="39" t="s">
-        <v>61</v>
-      </c>
-      <c r="E10" s="39" t="s">
-        <v>62</v>
-      </c>
-      <c r="F10" s="32">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="81.599999999999994" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="24" t="s">
-        <v>36</v>
-      </c>
-      <c r="B11" s="24" t="s">
-        <v>37</v>
-      </c>
-      <c r="C11" s="24" t="s">
-        <v>38</v>
-      </c>
-      <c r="D11" s="24" t="s">
-        <v>39</v>
-      </c>
-      <c r="E11" s="24" t="s">
-        <v>40</v>
-      </c>
-      <c r="F11" s="36">
-        <v>10</v>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A1:A3"/>
-    <mergeCell ref="B1:E1"/>
-    <mergeCell ref="F1:F3"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:C3"/>
-  </mergeCells>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -2887,10 +3727,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>4</v>
+        <v>66</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -2938,7 +3778,7 @@
         <v>2.5</v>
       </c>
       <c r="B7">
-        <v>1.1000000000000001</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="8" spans="1:2" x14ac:dyDescent="0.25">
@@ -2962,7 +3802,7 @@
         <v>4</v>
       </c>
       <c r="B10">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
@@ -2970,7 +3810,7 @@
         <v>4.5</v>
       </c>
       <c r="B11">
-        <v>1.2</v>
+        <v>1.3</v>
       </c>
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
@@ -2986,7 +3826,7 @@
         <v>5.5</v>
       </c>
       <c r="B13">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
@@ -2994,7 +3834,7 @@
         <v>6</v>
       </c>
       <c r="B14">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
@@ -3002,7 +3842,7 @@
         <v>6.5</v>
       </c>
       <c r="B15">
-        <v>1.3</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
@@ -3010,7 +3850,7 @@
         <v>7</v>
       </c>
       <c r="B16">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
@@ -3018,7 +3858,7 @@
         <v>7.5</v>
       </c>
       <c r="B17">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
@@ -3026,7 +3866,7 @@
         <v>8</v>
       </c>
       <c r="B18">
-        <v>1.4</v>
+        <v>1.5</v>
       </c>
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
@@ -3034,7 +3874,7 @@
         <v>8.5</v>
       </c>
       <c r="B19">
-        <v>1.4</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
@@ -3042,7 +3882,7 @@
         <v>9</v>
       </c>
       <c r="B20">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="21" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3050,7 +3890,7 @@
         <v>9.5</v>
       </c>
       <c r="B21">
-        <v>1.5</v>
+        <v>1.6</v>
       </c>
     </row>
     <row r="22" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3058,7 +3898,7 @@
         <v>10</v>
       </c>
       <c r="B22">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="23" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3066,7 +3906,7 @@
         <v>10.5</v>
       </c>
       <c r="B23">
-        <v>1.5</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="24" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3074,7 +3914,7 @@
         <v>11</v>
       </c>
       <c r="B24">
-        <v>1.6</v>
+        <v>1.7</v>
       </c>
     </row>
     <row r="25" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3082,7 +3922,7 @@
         <v>11.5</v>
       </c>
       <c r="B25">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="26" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3090,7 +3930,7 @@
         <v>12</v>
       </c>
       <c r="B26">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="27" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3098,7 +3938,7 @@
         <v>12.5</v>
       </c>
       <c r="B27">
-        <v>1.6</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="28" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3106,7 +3946,7 @@
         <v>13</v>
       </c>
       <c r="B28">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="29" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3114,7 +3954,7 @@
         <v>13.5</v>
       </c>
       <c r="B29">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="30" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3122,7 +3962,7 @@
         <v>14</v>
       </c>
       <c r="B30">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
     </row>
     <row r="31" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3130,7 +3970,7 @@
         <v>14.5</v>
       </c>
       <c r="B31">
-        <v>1.7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="32" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3138,7 +3978,7 @@
         <v>15</v>
       </c>
       <c r="B32">
-        <v>1.8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="33" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3146,7 +3986,7 @@
         <v>15.5</v>
       </c>
       <c r="B33">
-        <v>1.8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3154,7 +3994,7 @@
         <v>16</v>
       </c>
       <c r="B34">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="35" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3162,7 +4002,7 @@
         <v>16.5</v>
       </c>
       <c r="B35">
-        <v>1.8</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="36" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3170,7 +4010,7 @@
         <v>17</v>
       </c>
       <c r="B36">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
     </row>
     <row r="37" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3178,7 +4018,7 @@
         <v>17.5</v>
       </c>
       <c r="B37">
-        <v>1.9</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="38" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3186,7 +4026,7 @@
         <v>18</v>
       </c>
       <c r="B38">
-        <v>1.9</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="39" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3194,7 +4034,7 @@
         <v>18.5</v>
       </c>
       <c r="B39">
-        <v>1.9</v>
+        <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="40" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3202,7 +4042,7 @@
         <v>19</v>
       </c>
       <c r="B40">
-        <v>2</v>
+        <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="41" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3210,7 +4050,7 @@
         <v>19.5</v>
       </c>
       <c r="B41">
-        <v>2</v>
+        <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="42" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3218,7 +4058,7 @@
         <v>20</v>
       </c>
       <c r="B42">
-        <v>2</v>
+        <v>2.2999999999999998</v>
       </c>
     </row>
     <row r="43" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3226,7 +4066,7 @@
         <v>20.5</v>
       </c>
       <c r="B43">
-        <v>2</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="44" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3234,7 +4074,7 @@
         <v>21</v>
       </c>
       <c r="B44">
-        <v>2.1</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="45" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3242,7 +4082,7 @@
         <v>21.5</v>
       </c>
       <c r="B45">
-        <v>2.1</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="46" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3250,7 +4090,7 @@
         <v>22</v>
       </c>
       <c r="B46">
-        <v>2.1</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="47" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3258,7 +4098,7 @@
         <v>22.5</v>
       </c>
       <c r="B47">
-        <v>2.1</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="48" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3266,7 +4106,7 @@
         <v>23</v>
       </c>
       <c r="B48">
-        <v>2.2000000000000002</v>
+        <v>2.5</v>
       </c>
     </row>
     <row r="49" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3274,7 +4114,7 @@
         <v>23.5</v>
       </c>
       <c r="B49">
-        <v>2.2000000000000002</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="50" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3282,7 +4122,7 @@
         <v>24</v>
       </c>
       <c r="B50">
-        <v>2.2000000000000002</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="51" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3290,7 +4130,7 @@
         <v>24.5</v>
       </c>
       <c r="B51">
-        <v>2.2000000000000002</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="52" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3298,7 +4138,7 @@
         <v>25</v>
       </c>
       <c r="B52">
-        <v>2.2999999999999998</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="53" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3306,7 +4146,7 @@
         <v>25.5</v>
       </c>
       <c r="B53">
-        <v>2.2999999999999998</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="54" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3314,7 +4154,7 @@
         <v>26</v>
       </c>
       <c r="B54">
-        <v>2.2999999999999998</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="55" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3322,7 +4162,7 @@
         <v>26.5</v>
       </c>
       <c r="B55">
-        <v>2.2999999999999998</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="56" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3330,7 +4170,7 @@
         <v>27</v>
       </c>
       <c r="B56">
-        <v>2.4</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="57" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3338,7 +4178,7 @@
         <v>27.5</v>
       </c>
       <c r="B57">
-        <v>2.4</v>
+        <v>2.8</v>
       </c>
     </row>
     <row r="58" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3346,7 +4186,7 @@
         <v>28</v>
       </c>
       <c r="B58">
-        <v>2.4</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="59" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3354,7 +4194,7 @@
         <v>28.5</v>
       </c>
       <c r="B59">
-        <v>2.4</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="60" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3362,7 +4202,7 @@
         <v>29</v>
       </c>
       <c r="B60">
-        <v>2.5</v>
+        <v>2.9</v>
       </c>
     </row>
     <row r="61" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3370,7 +4210,7 @@
         <v>29.5</v>
       </c>
       <c r="B61">
-        <v>2.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="62" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3378,7 +4218,7 @@
         <v>30</v>
       </c>
       <c r="B62">
-        <v>2.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="63" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3386,7 +4226,7 @@
         <v>30.5</v>
       </c>
       <c r="B63">
-        <v>2.5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="64" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3394,7 +4234,7 @@
         <v>31</v>
       </c>
       <c r="B64">
-        <v>2.6</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="65" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3402,7 +4242,7 @@
         <v>31.5</v>
       </c>
       <c r="B65">
-        <v>2.6</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="66" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3410,7 +4250,7 @@
         <v>32</v>
       </c>
       <c r="B66">
-        <v>2.6</v>
+        <v>3.1</v>
       </c>
     </row>
     <row r="67" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3418,7 +4258,7 @@
         <v>32.5</v>
       </c>
       <c r="B67">
-        <v>2.6</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="68" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3426,7 +4266,7 @@
         <v>33</v>
       </c>
       <c r="B68">
-        <v>2.7</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="69" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3434,7 +4274,7 @@
         <v>33.5</v>
       </c>
       <c r="B69">
-        <v>2.7</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="70" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3442,7 +4282,7 @@
         <v>34</v>
       </c>
       <c r="B70">
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="71" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3450,7 +4290,7 @@
         <v>34.5</v>
       </c>
       <c r="B71">
-        <v>2.7</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="72" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3458,7 +4298,7 @@
         <v>35</v>
       </c>
       <c r="B72">
-        <v>2.8</v>
+        <v>3.3</v>
       </c>
     </row>
     <row r="73" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3466,7 +4306,7 @@
         <v>35.5</v>
       </c>
       <c r="B73">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="74" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3474,7 +4314,7 @@
         <v>36</v>
       </c>
       <c r="B74">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="75" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3482,7 +4322,7 @@
         <v>36.5</v>
       </c>
       <c r="B75">
-        <v>2.8</v>
+        <v>3.4</v>
       </c>
     </row>
     <row r="76" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3490,7 +4330,7 @@
         <v>37</v>
       </c>
       <c r="B76">
-        <v>2.9</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="77" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3498,7 +4338,7 @@
         <v>37.5</v>
       </c>
       <c r="B77">
-        <v>2.9</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="78" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3506,7 +4346,7 @@
         <v>38</v>
       </c>
       <c r="B78">
-        <v>2.9</v>
+        <v>3.5</v>
       </c>
     </row>
     <row r="79" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3514,7 +4354,7 @@
         <v>38.5</v>
       </c>
       <c r="B79">
-        <v>2.9</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="80" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3522,7 +4362,7 @@
         <v>39</v>
       </c>
       <c r="B80">
-        <v>3</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="81" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3530,7 +4370,7 @@
         <v>39.5</v>
       </c>
       <c r="B81">
-        <v>3</v>
+        <v>3.6</v>
       </c>
     </row>
     <row r="82" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3538,7 +4378,7 @@
         <v>40</v>
       </c>
       <c r="B82">
-        <v>3</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="83" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3546,7 +4386,7 @@
         <v>40.5</v>
       </c>
       <c r="B83">
-        <v>3</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="84" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3554,7 +4394,7 @@
         <v>41</v>
       </c>
       <c r="B84">
-        <v>3.1</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="85" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3562,7 +4402,7 @@
         <v>41.5</v>
       </c>
       <c r="B85">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="86" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3570,7 +4410,7 @@
         <v>42</v>
       </c>
       <c r="B86">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="87" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3578,7 +4418,7 @@
         <v>42.5</v>
       </c>
       <c r="B87">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="88" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3586,7 +4426,7 @@
         <v>43</v>
       </c>
       <c r="B88">
-        <v>3.2</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="89" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3594,7 +4434,7 @@
         <v>43.5</v>
       </c>
       <c r="B89">
-        <v>3.2</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="90" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3602,7 +4442,7 @@
         <v>44</v>
       </c>
       <c r="B90">
-        <v>3.2</v>
+        <v>3.9</v>
       </c>
     </row>
     <row r="91" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3610,7 +4450,7 @@
         <v>44.5</v>
       </c>
       <c r="B91">
-        <v>3.2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="92" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3618,7 +4458,7 @@
         <v>45</v>
       </c>
       <c r="B92">
-        <v>3.3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="93" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3626,7 +4466,7 @@
         <v>45.5</v>
       </c>
       <c r="B93">
-        <v>3.3</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="94" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3634,7 +4474,7 @@
         <v>46</v>
       </c>
       <c r="B94">
-        <v>3.3</v>
+        <v>4.0999999999999996</v>
       </c>
     </row>
     <row r="95" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3642,7 +4482,7 @@
         <v>46.5</v>
       </c>
       <c r="B95">
-        <v>3.3</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="96" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3650,7 +4490,7 @@
         <v>47</v>
       </c>
       <c r="B96">
-        <v>3.4</v>
+        <v>4.2</v>
       </c>
     </row>
     <row r="97" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3658,7 +4498,7 @@
         <v>47.5</v>
       </c>
       <c r="B97">
-        <v>3.4</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="98" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3666,7 +4506,7 @@
         <v>48</v>
       </c>
       <c r="B98">
-        <v>3.4</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="99" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3674,7 +4514,7 @@
         <v>48.5</v>
       </c>
       <c r="B99">
-        <v>3.4</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="100" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3682,7 +4522,7 @@
         <v>49</v>
       </c>
       <c r="B100">
-        <v>3.5</v>
+        <v>4.4000000000000004</v>
       </c>
     </row>
     <row r="101" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3690,7 +4530,7 @@
         <v>49.5</v>
       </c>
       <c r="B101">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="102" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3698,7 +4538,7 @@
         <v>50</v>
       </c>
       <c r="B102">
-        <v>3.5</v>
+        <v>4.5</v>
       </c>
     </row>
     <row r="103" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3706,7 +4546,7 @@
         <v>50.5</v>
       </c>
       <c r="B103">
-        <v>3.5</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="104" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3714,7 +4554,7 @@
         <v>51</v>
       </c>
       <c r="B104">
-        <v>3.6</v>
+        <v>4.5999999999999996</v>
       </c>
     </row>
     <row r="105" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3722,7 +4562,7 @@
         <v>51.5</v>
       </c>
       <c r="B105">
-        <v>3.6</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="106" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3730,7 +4570,7 @@
         <v>52</v>
       </c>
       <c r="B106">
-        <v>3.6</v>
+        <v>4.7</v>
       </c>
     </row>
     <row r="107" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3738,7 +4578,7 @@
         <v>52.5</v>
       </c>
       <c r="B107">
-        <v>3.6</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="108" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3746,7 +4586,7 @@
         <v>53</v>
       </c>
       <c r="B108">
-        <v>3.7</v>
+        <v>4.8</v>
       </c>
     </row>
     <row r="109" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3754,7 +4594,7 @@
         <v>53.5</v>
       </c>
       <c r="B109">
-        <v>3.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="110" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3762,7 +4602,7 @@
         <v>54</v>
       </c>
       <c r="B110">
-        <v>3.7</v>
+        <v>4.9000000000000004</v>
       </c>
     </row>
     <row r="111" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3770,7 +4610,7 @@
         <v>54.5</v>
       </c>
       <c r="B111">
-        <v>3.7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="112" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3778,7 +4618,7 @@
         <v>55</v>
       </c>
       <c r="B112">
-        <v>3.8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="113" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3786,7 +4626,7 @@
         <v>55.5</v>
       </c>
       <c r="B113">
-        <v>3.8</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="114" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3794,7 +4634,7 @@
         <v>56</v>
       </c>
       <c r="B114">
-        <v>3.8</v>
+        <v>5.0999999999999996</v>
       </c>
     </row>
     <row r="115" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3802,7 +4642,7 @@
         <v>56.5</v>
       </c>
       <c r="B115">
-        <v>3.8</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="116" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3810,7 +4650,7 @@
         <v>57</v>
       </c>
       <c r="B116">
-        <v>3.9</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="117" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3818,7 +4658,7 @@
         <v>57.5</v>
       </c>
       <c r="B117">
-        <v>3.9</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="118" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3826,7 +4666,7 @@
         <v>58</v>
       </c>
       <c r="B118">
-        <v>3.9</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="119" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3834,7 +4674,7 @@
         <v>58.5</v>
       </c>
       <c r="B119">
-        <v>3.9</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="120" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3842,7 +4682,7 @@
         <v>59</v>
       </c>
       <c r="B120">
-        <v>4</v>
+        <v>5.4</v>
       </c>
     </row>
     <row r="121" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3850,7 +4690,7 @@
         <v>59.5</v>
       </c>
       <c r="B121">
-        <v>4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="122" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3858,7 +4698,7 @@
         <v>60</v>
       </c>
       <c r="B122">
-        <v>4</v>
+        <v>5.5</v>
       </c>
     </row>
     <row r="123" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3866,7 +4706,7 @@
         <v>60.5</v>
       </c>
       <c r="B123">
-        <v>4</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="124" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3874,7 +4714,7 @@
         <v>61</v>
       </c>
       <c r="B124">
-        <v>4.0999999999999996</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="125" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3882,7 +4722,7 @@
         <v>61.5</v>
       </c>
       <c r="B125">
-        <v>4.0999999999999996</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="126" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3890,7 +4730,7 @@
         <v>62</v>
       </c>
       <c r="B126">
-        <v>4.2</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="127" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3898,7 +4738,7 @@
         <v>62.5</v>
       </c>
       <c r="B127">
-        <v>4.2</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="128" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3906,7 +4746,7 @@
         <v>63</v>
       </c>
       <c r="B128">
-        <v>4.2</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="129" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3914,7 +4754,7 @@
         <v>63.5</v>
       </c>
       <c r="B129">
-        <v>4.3</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="130" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3922,7 +4762,7 @@
         <v>64</v>
       </c>
       <c r="B130">
-        <v>4.3</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="131" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3930,7 +4770,7 @@
         <v>64.5</v>
       </c>
       <c r="B131">
-        <v>4.3</v>
+        <v>6</v>
       </c>
     </row>
     <row r="132" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3938,7 +4778,7 @@
         <v>65</v>
       </c>
       <c r="B132">
-        <v>4.4000000000000004</v>
+        <v>6</v>
       </c>
     </row>
     <row r="133" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3946,7 +4786,7 @@
         <v>65.5</v>
       </c>
       <c r="B133">
-        <v>4.4000000000000004</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="134" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3954,7 +4794,7 @@
         <v>66</v>
       </c>
       <c r="B134">
-        <v>4.5</v>
+        <v>6.1</v>
       </c>
     </row>
     <row r="135" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3962,7 +4802,7 @@
         <v>66.5</v>
       </c>
       <c r="B135">
-        <v>4.5</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="136" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3970,7 +4810,7 @@
         <v>67</v>
       </c>
       <c r="B136">
-        <v>4.5</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="137" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3978,7 +4818,7 @@
         <v>67.5</v>
       </c>
       <c r="B137">
-        <v>4.5999999999999996</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="138" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3986,7 +4826,7 @@
         <v>68</v>
       </c>
       <c r="B138">
-        <v>4.5999999999999996</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="139" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -3994,7 +4834,7 @@
         <v>68.5</v>
       </c>
       <c r="B139">
-        <v>4.5999999999999996</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="140" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4002,7 +4842,7 @@
         <v>69</v>
       </c>
       <c r="B140">
-        <v>4.7</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="141" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4010,7 +4850,7 @@
         <v>69.5</v>
       </c>
       <c r="B141">
-        <v>4.7</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="142" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4018,7 +4858,7 @@
         <v>70</v>
       </c>
       <c r="B142">
-        <v>4.8</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="143" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4026,7 +4866,7 @@
         <v>70.5</v>
       </c>
       <c r="B143">
-        <v>4.8</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="144" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4034,7 +4874,7 @@
         <v>71</v>
       </c>
       <c r="B144">
-        <v>4.8</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="145" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4042,7 +4882,7 @@
         <v>71.5</v>
       </c>
       <c r="B145">
-        <v>4.9000000000000004</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="146" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4050,7 +4890,7 @@
         <v>72</v>
       </c>
       <c r="B146">
-        <v>4.9000000000000004</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="147" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4058,7 +4898,7 @@
         <v>72.5</v>
       </c>
       <c r="B147">
-        <v>4.9000000000000004</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="148" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4066,7 +4906,7 @@
         <v>73</v>
       </c>
       <c r="B148">
-        <v>5</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="149" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4074,7 +4914,7 @@
         <v>73.5</v>
       </c>
       <c r="B149">
-        <v>5</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="150" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4082,7 +4922,7 @@
         <v>74</v>
       </c>
       <c r="B150">
-        <v>5.0999999999999996</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="151" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4090,7 +4930,7 @@
         <v>74.5</v>
       </c>
       <c r="B151">
-        <v>5.0999999999999996</v>
+        <v>7</v>
       </c>
     </row>
     <row r="152" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -4098,415 +4938,65 @@
         <v>75</v>
       </c>
       <c r="B152">
-        <v>5.0999999999999996</v>
-      </c>
-    </row>
-    <row r="153" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A153">
-        <v>75.5</v>
-      </c>
-      <c r="B153">
-        <v>5.2</v>
-      </c>
-    </row>
-    <row r="154" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A154">
-        <v>76</v>
-      </c>
-      <c r="B154">
-        <v>5.2</v>
-      </c>
-    </row>
-    <row r="155" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A155">
-        <v>76.5</v>
-      </c>
-      <c r="B155">
-        <v>5.2</v>
-      </c>
-    </row>
-    <row r="156" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A156">
-        <v>77</v>
-      </c>
-      <c r="B156">
-        <v>5.3</v>
-      </c>
-    </row>
-    <row r="157" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A157">
-        <v>77.5</v>
-      </c>
-      <c r="B157">
-        <v>5.3</v>
-      </c>
-    </row>
-    <row r="158" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A158">
-        <v>78</v>
-      </c>
-      <c r="B158">
-        <v>5.4</v>
-      </c>
-    </row>
-    <row r="159" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A159">
-        <v>78.5</v>
-      </c>
-      <c r="B159">
-        <v>5.4</v>
-      </c>
-    </row>
-    <row r="160" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A160">
-        <v>79</v>
-      </c>
-      <c r="B160">
-        <v>5.4</v>
-      </c>
-    </row>
-    <row r="161" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A161">
-        <v>79.5</v>
-      </c>
-      <c r="B161">
-        <v>5.5</v>
-      </c>
-    </row>
-    <row r="162" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A162">
-        <v>80</v>
-      </c>
-      <c r="B162">
-        <v>5.5</v>
-      </c>
-    </row>
-    <row r="163" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A163">
-        <v>80.5</v>
-      </c>
-      <c r="B163">
-        <v>5.5</v>
-      </c>
-    </row>
-    <row r="164" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A164">
-        <v>81</v>
-      </c>
-      <c r="B164">
-        <v>5.6</v>
-      </c>
-    </row>
-    <row r="165" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A165">
-        <v>81.5</v>
-      </c>
-      <c r="B165">
-        <v>5.6</v>
-      </c>
-    </row>
-    <row r="166" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A166">
-        <v>82</v>
-      </c>
-      <c r="B166">
-        <v>5.7</v>
-      </c>
-    </row>
-    <row r="167" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A167">
-        <v>82.5</v>
-      </c>
-      <c r="B167">
-        <v>5.7</v>
-      </c>
-    </row>
-    <row r="168" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A168">
-        <v>83</v>
-      </c>
-      <c r="B168">
-        <v>5.7</v>
-      </c>
-    </row>
-    <row r="169" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A169">
-        <v>83.5</v>
-      </c>
-      <c r="B169">
-        <v>5.8</v>
-      </c>
-    </row>
-    <row r="170" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A170">
-        <v>84</v>
-      </c>
-      <c r="B170">
-        <v>5.8</v>
-      </c>
-    </row>
-    <row r="171" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A171">
-        <v>84.5</v>
-      </c>
-      <c r="B171">
-        <v>5.8</v>
-      </c>
-    </row>
-    <row r="172" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A172">
-        <v>85</v>
-      </c>
-      <c r="B172">
-        <v>5.9</v>
-      </c>
-    </row>
-    <row r="173" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A173">
-        <v>85.5</v>
-      </c>
-      <c r="B173">
-        <v>5.9</v>
-      </c>
-    </row>
-    <row r="174" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A174">
-        <v>86</v>
-      </c>
-      <c r="B174">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="175" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A175">
-        <v>86.5</v>
-      </c>
-      <c r="B175">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="176" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A176">
-        <v>87</v>
-      </c>
-      <c r="B176">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="177" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A177">
-        <v>87.5</v>
-      </c>
-      <c r="B177">
-        <v>6.1</v>
-      </c>
-    </row>
-    <row r="178" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A178">
-        <v>88</v>
-      </c>
-      <c r="B178">
-        <v>6.1</v>
-      </c>
-    </row>
-    <row r="179" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A179">
-        <v>88.5</v>
-      </c>
-      <c r="B179">
-        <v>6.1</v>
-      </c>
-    </row>
-    <row r="180" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A180">
-        <v>89</v>
-      </c>
-      <c r="B180">
-        <v>6.2</v>
-      </c>
-    </row>
-    <row r="181" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A181">
-        <v>89.5</v>
-      </c>
-      <c r="B181">
-        <v>6.2</v>
-      </c>
-    </row>
-    <row r="182" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A182">
-        <v>90</v>
-      </c>
-      <c r="B182">
-        <v>6.3</v>
-      </c>
-    </row>
-    <row r="183" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A183">
-        <v>90.5</v>
-      </c>
-      <c r="B183">
-        <v>6.3</v>
-      </c>
-    </row>
-    <row r="184" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A184">
-        <v>91</v>
-      </c>
-      <c r="B184">
-        <v>6.3</v>
-      </c>
-    </row>
-    <row r="185" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A185">
-        <v>91.5</v>
-      </c>
-      <c r="B185">
-        <v>6.4</v>
-      </c>
-    </row>
-    <row r="186" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A186">
-        <v>92</v>
-      </c>
-      <c r="B186">
-        <v>6.4</v>
-      </c>
-    </row>
-    <row r="187" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A187">
-        <v>92.5</v>
-      </c>
-      <c r="B187">
-        <v>6.4</v>
-      </c>
-    </row>
-    <row r="188" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A188">
-        <v>93</v>
-      </c>
-      <c r="B188">
-        <v>6.5</v>
-      </c>
-    </row>
-    <row r="189" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A189">
-        <v>93.5</v>
-      </c>
-      <c r="B189">
-        <v>6.5</v>
-      </c>
-    </row>
-    <row r="190" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A190">
-        <v>94</v>
-      </c>
-      <c r="B190">
-        <v>6.6</v>
-      </c>
-    </row>
-    <row r="191" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A191">
-        <v>94.5</v>
-      </c>
-      <c r="B191">
-        <v>6.6</v>
-      </c>
-    </row>
-    <row r="192" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A192">
-        <v>95</v>
-      </c>
-      <c r="B192">
-        <v>6.6</v>
-      </c>
-    </row>
-    <row r="193" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A193">
-        <v>95.5</v>
-      </c>
-      <c r="B193">
-        <v>6.7</v>
-      </c>
-    </row>
-    <row r="194" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A194">
-        <v>96</v>
-      </c>
-      <c r="B194">
-        <v>6.7</v>
-      </c>
-    </row>
-    <row r="195" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A195">
-        <v>96.5</v>
-      </c>
-      <c r="B195">
-        <v>6.7</v>
-      </c>
-    </row>
-    <row r="196" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A196">
-        <v>97</v>
-      </c>
-      <c r="B196">
-        <v>6.8</v>
-      </c>
-    </row>
-    <row r="197" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A197">
-        <v>97.5</v>
-      </c>
-      <c r="B197">
-        <v>6.8</v>
-      </c>
-    </row>
-    <row r="198" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A198">
-        <v>98</v>
-      </c>
-      <c r="B198">
-        <v>6.9</v>
-      </c>
-    </row>
-    <row r="199" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A199">
-        <v>98.5</v>
-      </c>
-      <c r="B199">
-        <v>6.9</v>
-      </c>
-    </row>
-    <row r="200" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A200">
-        <v>99</v>
-      </c>
-      <c r="B200">
-        <v>6.9</v>
-      </c>
-    </row>
-    <row r="201" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A201">
-        <v>99.5</v>
-      </c>
-      <c r="B201">
         <v>7</v>
       </c>
     </row>
-    <row r="202" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A202">
-        <v>100</v>
-      </c>
-      <c r="B202">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="203" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="204" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="205" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="206" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="207" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="208" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="153" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="154" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="155" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="156" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="157" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="158" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="159" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="160" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="161" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="162" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="163" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="164" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="165" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="166" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="167" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="168" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="169" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="170" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="171" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="172" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="173" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="174" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="175" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="176" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="177" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="178" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="179" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="180" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="181" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="182" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="183" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="184" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="185" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="186" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="187" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="188" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="189" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="190" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="191" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="192" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="193" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="194" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="195" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="196" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="197" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="198" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="199" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="200" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="201" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="202" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="203" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="204" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="205" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="206" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="207" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="208" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="209" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="210" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="211" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -5315,10 +5805,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>71</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -6707,10 +7197,10 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>4</v>
+        <v>66</v>
       </c>
       <c r="B1" t="s">
-        <v>13</v>
+        <v>67</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
@@ -8088,34 +8578,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="57" t="s">
-        <v>3</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>4</v>
-      </c>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="8"/>
+      <c r="A1" s="71" t="s">
+        <v>73</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>66</v>
+      </c>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="9"/>
     </row>
     <row r="2" spans="1:5" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="58"/>
-      <c r="B2" s="9" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="10" t="s">
+      <c r="A2" s="72"/>
+      <c r="B2" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>64</v>
+      </c>
+      <c r="D2" s="31" t="s">
+        <v>74</v>
+      </c>
+      <c r="E2" s="50" t="s">
         <v>6</v>
-      </c>
-      <c r="D2" s="29" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" s="11" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:5" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A3" s="12" t="s">
-        <v>8</v>
+        <v>75</v>
       </c>
       <c r="B3" s="13">
         <v>4</v>

</xml_diff>